<commit_message>
problems with missing types
</commit_message>
<xml_diff>
--- a/Results/table2latex.xlsx
+++ b/Results/table2latex.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbueren\Google Drive\endo_health\metric_model\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E012D12F-1E3E-46B3-B5A3-BE69EF1997F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71DE7C36-ACEA-43FA-A795-AD3C59EF2988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4D131852-BDAB-48D2-B0B4-24C9607E5D25}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{4D131852-BDAB-48D2-B0B4-24C9607E5D25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="59">
   <si>
     <t>Protective</t>
   </si>
@@ -77,15 +77,6 @@
   </si>
   <si>
     <t>ans</t>
-  </si>
-  <si>
-    <t>=</t>
-  </si>
-  <si>
-    <t>Edu gradient</t>
-  </si>
-  <si>
-    <t>Gender gap</t>
   </si>
   <si>
     <t>H</t>
@@ -156,15 +147,82 @@
   <si>
     <t xml:space="preserve">\\ </t>
   </si>
+  <si>
+    <t xml:space="preserve">\multicolumn{2}{c}{All} </t>
+  </si>
+  <si>
+    <t>\textsc{pro}</t>
+  </si>
+  <si>
+    <t>\textsc{det}</t>
+  </si>
+  <si>
+    <t>pr(e)</t>
+  </si>
+  <si>
+    <t>hsd</t>
+  </si>
+  <si>
+    <t>hsg</t>
+  </si>
+  <si>
+    <t>cg</t>
+  </si>
+  <si>
+    <t>pr(pro)</t>
+  </si>
+  <si>
+    <t>pr(det)</t>
+  </si>
+  <si>
+    <t>pr(hsd|pro)</t>
+  </si>
+  <si>
+    <t>pr(hsg|pro)</t>
+  </si>
+  <si>
+    <t>pr(cg|pro)</t>
+  </si>
+  <si>
+    <t>LE_pro</t>
+  </si>
+  <si>
+    <t>av_le</t>
+  </si>
+  <si>
+    <t>LE_det</t>
+  </si>
+  <si>
+    <t>Av le hsd</t>
+  </si>
+  <si>
+    <t>Av le cg</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>$=$ht</t>
+  </si>
+  <si>
+    <t>$=$y</t>
+  </si>
+  <si>
+    <t>Pr(e)</t>
+  </si>
+  <si>
+    <t>Pr(det|e)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -218,7 +276,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -229,6 +287,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2438,16 +2497,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F330EFCA-C7DF-4136-98BB-2504A28BB96C}">
-  <dimension ref="A2:AP79"/>
+  <dimension ref="A2:AT79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="15" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="2.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5.28515625" customWidth="1"/>
     <col min="26" max="26" width="28.42578125" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="2.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="7.140625" customWidth="1"/>
     <col min="29" max="29" width="2.42578125" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="30.85546875" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="2.42578125" bestFit="1" customWidth="1"/>
@@ -2476,16 +2536,16 @@
         <v>9.3678000000000008</v>
       </c>
       <c r="M2">
-        <v>0.42859999999999998</v>
+        <v>0.44309999999999999</v>
       </c>
       <c r="N2">
-        <v>28.956800000000001</v>
+        <v>28.5366</v>
       </c>
       <c r="O2">
-        <v>17.529399999999999</v>
+        <v>17.219799999999999</v>
       </c>
       <c r="P2">
-        <v>11.4274</v>
+        <v>11.3169</v>
       </c>
       <c r="S2">
         <v>0.42859999999999998</v>
@@ -2498,6 +2558,9 @@
       </c>
       <c r="V2">
         <v>11.4274</v>
+      </c>
+      <c r="X2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
@@ -2514,16 +2577,16 @@
         <v>10.9596</v>
       </c>
       <c r="M3">
-        <v>0.57140000000000002</v>
+        <v>0.55689999999999995</v>
       </c>
       <c r="N3">
-        <v>21.393799999999999</v>
+        <v>21.9603</v>
       </c>
       <c r="O3">
-        <v>11.8089</v>
+        <v>12.2713</v>
       </c>
       <c r="P3">
-        <v>9.5847999999999995</v>
+        <v>9.6890000000000001</v>
       </c>
       <c r="S3">
         <v>0.57140000000000002</v>
@@ -2536,6 +2599,12 @@
       </c>
       <c r="V3">
         <v>9.5847999999999995</v>
+      </c>
+      <c r="X3" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y3">
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
@@ -2552,16 +2621,16 @@
         <v>5.7394999999999996</v>
       </c>
       <c r="M4">
-        <v>0.67859999999999998</v>
+        <v>0.68959999999999999</v>
       </c>
       <c r="N4">
-        <v>30.261800000000001</v>
+        <v>30.138300000000001</v>
       </c>
       <c r="O4">
-        <v>23.8552</v>
+        <v>23.950700000000001</v>
       </c>
       <c r="P4">
-        <v>6.4066000000000001</v>
+        <v>6.1875</v>
       </c>
       <c r="S4">
         <v>0.67859999999999998</v>
@@ -2574,6 +2643,12 @@
       </c>
       <c r="V4">
         <v>6.4066000000000001</v>
+      </c>
+      <c r="X4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y4">
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
@@ -2590,16 +2665,16 @@
         <v>5.9078999999999997</v>
       </c>
       <c r="M5">
-        <v>0.32140000000000002</v>
+        <v>0.31040000000000001</v>
       </c>
       <c r="N5">
-        <v>23.019400000000001</v>
+        <v>23.289100000000001</v>
       </c>
       <c r="O5">
-        <v>16.190300000000001</v>
+        <v>16.069099999999999</v>
       </c>
       <c r="P5">
-        <v>6.8291000000000004</v>
+        <v>7.2199</v>
       </c>
       <c r="S5">
         <v>0.32140000000000002</v>
@@ -2612,6 +2687,13 @@
       </c>
       <c r="V5">
         <v>6.8291000000000004</v>
+      </c>
+      <c r="X5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y5">
+        <f>100-Y4-Y3</f>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -2628,16 +2710,16 @@
         <v>4.0126999999999997</v>
       </c>
       <c r="M6">
-        <v>0.91590000000000005</v>
+        <v>0.93600000000000005</v>
       </c>
       <c r="N6">
-        <v>33.386800000000001</v>
+        <v>33.424700000000001</v>
       </c>
       <c r="O6">
-        <v>29.600899999999999</v>
+        <v>29.8184</v>
       </c>
       <c r="P6">
-        <v>3.7858999999999998</v>
+        <v>3.6063000000000001</v>
       </c>
       <c r="S6">
         <v>0.91590000000000005</v>
@@ -2650,6 +2732,13 @@
       </c>
       <c r="V6">
         <v>3.7858999999999998</v>
+      </c>
+      <c r="X6" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y6">
+        <f>AF21*Y3/100+AJ21*Y4/100+AN21*Y5/100</f>
+        <v>29.300209970200001</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -2666,16 +2755,16 @@
         <v>3.3725999999999998</v>
       </c>
       <c r="M7">
-        <v>8.4099999999999994E-2</v>
+        <v>6.4000000000000001E-2</v>
       </c>
       <c r="N7">
-        <v>24.4633</v>
+        <v>23.822600000000001</v>
       </c>
       <c r="O7">
-        <v>19.1035</v>
+        <v>17.418600000000001</v>
       </c>
       <c r="P7">
-        <v>5.3597999999999999</v>
+        <v>6.4039999999999999</v>
       </c>
       <c r="S7">
         <v>8.4099999999999994E-2</v>
@@ -2704,16 +2793,16 @@
         <v>11.552</v>
       </c>
       <c r="M8">
-        <v>0.5544</v>
+        <v>0.54879999999999995</v>
       </c>
       <c r="N8">
-        <v>30.3338</v>
+        <v>30.038399999999999</v>
       </c>
       <c r="O8">
-        <v>15.0909</v>
+        <v>15.1334</v>
       </c>
       <c r="P8">
-        <v>15.242900000000001</v>
+        <v>14.904999999999999</v>
       </c>
       <c r="S8">
         <v>0.5544</v>
@@ -2726,6 +2815,13 @@
       </c>
       <c r="V8">
         <v>15.242900000000001</v>
+      </c>
+      <c r="X8" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y8">
+        <f>(AD22/100*Y3/100+AH22/100*Y4/100+AL22/100*Y5/100)*100</f>
+        <v>74.379400000000004</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -2742,16 +2838,16 @@
         <v>13.2494</v>
       </c>
       <c r="M9">
-        <v>0.4456</v>
+        <v>0.45119999999999999</v>
       </c>
       <c r="N9">
-        <v>23.210699999999999</v>
+        <v>23.815100000000001</v>
       </c>
       <c r="O9">
-        <v>9.9444999999999997</v>
+        <v>10.379899999999999</v>
       </c>
       <c r="P9">
-        <v>13.2662</v>
+        <v>13.4352</v>
       </c>
       <c r="S9">
         <v>0.4456</v>
@@ -2764,6 +2860,13 @@
       </c>
       <c r="V9">
         <v>13.2662</v>
+      </c>
+      <c r="X9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9">
+        <f>100-Y8</f>
+        <v>25.620599999999996</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -2780,16 +2883,16 @@
         <v>7.1492000000000004</v>
       </c>
       <c r="M10">
-        <v>0.71779999999999999</v>
+        <v>0.72419999999999995</v>
       </c>
       <c r="N10">
-        <v>33.219099999999997</v>
+        <v>33.209099999999999</v>
       </c>
       <c r="O10">
-        <v>25.819900000000001</v>
+        <v>26.057200000000002</v>
       </c>
       <c r="P10">
-        <v>7.3992000000000004</v>
+        <v>7.1519000000000004</v>
       </c>
       <c r="S10">
         <v>0.71779999999999999</v>
@@ -2802,6 +2905,10 @@
       </c>
       <c r="V10">
         <v>7.3992000000000004</v>
+      </c>
+      <c r="Y10">
+        <f>Y8-Y9</f>
+        <v>48.758800000000008</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -2818,16 +2925,16 @@
         <v>6.9217000000000004</v>
       </c>
       <c r="M11">
-        <v>0.28220000000000001</v>
+        <v>0.27579999999999999</v>
       </c>
       <c r="N11">
-        <v>26.0535</v>
+        <v>25.952400000000001</v>
       </c>
       <c r="O11">
-        <v>17.647300000000001</v>
+        <v>16.8109</v>
       </c>
       <c r="P11">
-        <v>8.4062000000000001</v>
+        <v>9.1415000000000006</v>
       </c>
       <c r="S11">
         <v>0.28220000000000001</v>
@@ -2856,16 +2963,16 @@
         <v>4.8164999999999996</v>
       </c>
       <c r="M12">
-        <v>0.92710000000000004</v>
+        <v>0.93610000000000004</v>
       </c>
       <c r="N12">
-        <v>34.942599999999999</v>
+        <v>34.973700000000001</v>
       </c>
       <c r="O12">
-        <v>30.402899999999999</v>
+        <v>30.670500000000001</v>
       </c>
       <c r="P12">
-        <v>4.5396999999999998</v>
+        <v>4.3032000000000004</v>
       </c>
       <c r="S12">
         <v>0.92710000000000004</v>
@@ -2878,6 +2985,13 @@
       </c>
       <c r="V12">
         <v>4.5396999999999998</v>
+      </c>
+      <c r="X12" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y12">
+        <f>AD22/100*Y3/100/(Y8/100)*100</f>
+        <v>8.3402124781861637</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -2894,16 +3008,16 @@
         <v>4.1228999999999996</v>
       </c>
       <c r="M13">
-        <v>7.2900000000000006E-2</v>
+        <v>6.3899999999999998E-2</v>
       </c>
       <c r="N13">
-        <v>28.201499999999999</v>
+        <v>27.5351</v>
       </c>
       <c r="O13">
-        <v>20.847899999999999</v>
+        <v>18.8123</v>
       </c>
       <c r="P13">
-        <v>7.3536000000000001</v>
+        <v>8.7227999999999994</v>
       </c>
       <c r="S13">
         <v>7.2900000000000006E-2</v>
@@ -2917,14 +3031,37 @@
       <c r="V13">
         <v>7.3536000000000001</v>
       </c>
+      <c r="X13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y13">
+        <f>AH22/100*Y4/100/(Y8/100)*100</f>
+        <v>46.356921405658014</v>
+      </c>
       <c r="AH13">
         <v>6.2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="X14" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y14">
+        <f>100-Y13-Y12</f>
+        <v>45.302866116155826</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
+      <c r="X15" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y15">
+        <f>AF22*Y12/100+AJ22*Y13/100+AN22*Y14/100</f>
+        <v>31.49354820877824</v>
+      </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -2961,8 +3098,15 @@
       <c r="J16" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="X16" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y16">
+        <f>(Y6-Y8/100*Y15)*100/Y9</f>
+        <v>22.932709514219013</v>
+      </c>
+    </row>
+    <row r="17" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>0</v>
       </c>
@@ -2997,8 +3141,12 @@
       <c r="J17" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="Y17">
+        <f>Y15-Y16</f>
+        <v>8.5608386945592265</v>
+      </c>
+    </row>
+    <row r="18" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -3034,7 +3182,7 @@
       </c>
       <c r="O18" s="2"/>
     </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>12</v>
       </c>
@@ -3044,38 +3192,44 @@
       <c r="I19" s="2"/>
       <c r="J19" s="3"/>
       <c r="M19" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="Q19" s="2"/>
       <c r="Y19" t="s">
         <v>3</v>
       </c>
       <c r="Z19" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="AC19" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD19" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="AG19" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH19" t="s">
-        <v>23</v>
-      </c>
-      <c r="AK19" s="3" t="s">
-        <v>3</v>
+        <v>19</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>9</v>
       </c>
       <c r="AL19" t="s">
-        <v>28</v>
-      </c>
-      <c r="AO19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AO19" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP19" t="s">
+        <v>25</v>
+      </c>
+      <c r="AS19" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -3118,88 +3272,100 @@
       </c>
       <c r="O20" s="2">
         <f>M2*100</f>
-        <v>42.86</v>
+        <v>44.31</v>
       </c>
       <c r="P20" t="s">
         <v>3</v>
       </c>
       <c r="Q20" s="2">
         <f>N2</f>
-        <v>28.956800000000001</v>
+        <v>28.5366</v>
       </c>
       <c r="R20" t="s">
         <v>9</v>
       </c>
       <c r="S20" s="2">
         <f>O2</f>
-        <v>17.529399999999999</v>
+        <v>17.219799999999999</v>
       </c>
       <c r="T20" t="s">
         <v>9</v>
       </c>
       <c r="U20" s="2">
         <f>P2</f>
-        <v>11.4274</v>
+        <v>11.3169</v>
       </c>
       <c r="V20" s="3" t="s">
         <v>4</v>
       </c>
       <c r="X20" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="Y20" t="s">
         <v>3</v>
       </c>
       <c r="Z20" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AA20" t="s">
         <v>3</v>
       </c>
       <c r="AB20" t="s">
+        <v>23</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>23</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>23</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>9</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>22</v>
+      </c>
+      <c r="AM20" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN20" t="s">
+        <v>23</v>
+      </c>
+      <c r="AO20" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP20" t="s">
+        <v>23</v>
+      </c>
+      <c r="AQ20" t="s">
+        <v>3</v>
+      </c>
+      <c r="AR20" t="s">
         <v>26</v>
       </c>
-      <c r="AC20" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD20" t="s">
-        <v>25</v>
-      </c>
-      <c r="AE20" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF20" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG20" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH20" t="s">
-        <v>25</v>
-      </c>
-      <c r="AI20" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ20" t="s">
-        <v>26</v>
-      </c>
-      <c r="AK20" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL20" t="s">
-        <v>26</v>
-      </c>
-      <c r="AM20" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN20" t="s">
-        <v>29</v>
-      </c>
-      <c r="AO20" s="3" t="s">
+      <c r="AS20" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>0</v>
       </c>
@@ -3242,34 +3408,34 @@
       </c>
       <c r="O21" s="2">
         <f>M3*100</f>
-        <v>57.14</v>
+        <v>55.69</v>
       </c>
       <c r="P21" t="s">
         <v>3</v>
       </c>
       <c r="Q21" s="2">
         <f>N3</f>
-        <v>21.393799999999999</v>
+        <v>21.9603</v>
       </c>
       <c r="R21" t="s">
         <v>9</v>
       </c>
       <c r="S21" s="2">
         <f>O3</f>
-        <v>11.8089</v>
+        <v>12.2713</v>
       </c>
       <c r="T21" t="s">
         <v>9</v>
       </c>
       <c r="U21" s="2">
         <f>P3</f>
-        <v>9.5847999999999995</v>
+        <v>9.6890000000000001</v>
       </c>
       <c r="V21" s="3" t="s">
         <v>4</v>
       </c>
       <c r="X21" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Y21" t="s">
         <v>3</v>
@@ -3280,12 +3446,11 @@
       <c r="AA21" t="s">
         <v>3</v>
       </c>
-      <c r="AB21" s="2">
-        <f>Z22/100*AB22+Z23/100*AB23</f>
-        <v>27.270251000000002</v>
+      <c r="AB21" t="s">
+        <v>10</v>
       </c>
       <c r="AC21" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD21">
         <v>100</v>
@@ -3295,10 +3460,10 @@
       </c>
       <c r="AF21" s="2">
         <f>AD22/100*AF22+AD23/100*AF23</f>
-        <v>27.934092640000003</v>
+        <v>24.874258529999999</v>
       </c>
       <c r="AG21" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH21">
         <v>100</v>
@@ -3308,31 +3473,44 @@
       </c>
       <c r="AJ21" s="2">
         <f>AH22/100*AJ22+AH23/100*AJ23</f>
-        <v>32.449832499999999</v>
-      </c>
-      <c r="AK21" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL21" s="2">
-        <f>AJ21-AB21</f>
-        <v>5.1795814999999976</v>
+        <v>28.012308320000002</v>
+      </c>
+      <c r="AK21" t="s">
+        <v>9</v>
+      </c>
+      <c r="AL21">
+        <v>100</v>
       </c>
       <c r="AM21" t="s">
         <v>3</v>
       </c>
       <c r="AN21" s="2">
-        <f>AJ21-(AB22*AH22/100+AB23*AH23/100)</f>
-        <v>4.2871474999999997</v>
-      </c>
-      <c r="AO21" s="3" t="s">
+        <f>AL22/100*AN22+AL23/100*AN23</f>
+        <v>32.810165599999998</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP21" s="2">
+        <f>AN21-AF21</f>
+        <v>7.935907069999999</v>
+      </c>
+      <c r="AQ21" t="s">
+        <v>3</v>
+      </c>
+      <c r="AR21" s="2">
+        <f>AN21-(AF22*AL22/100+AF23*AL23/100)</f>
+        <v>4.6944488</v>
+      </c>
+      <c r="AS21" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="AP21" s="7">
-        <f>(AL21-AN21)/AL21</f>
-        <v>0.17229847623789651</v>
-      </c>
-    </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="AT21" s="7">
+        <f>(AP21-AR21)/AP21</f>
+        <v>0.40845466578781392</v>
+      </c>
+    </row>
+    <row r="22" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>2</v>
       </c>
@@ -3367,100 +3545,112 @@
         <v>4</v>
       </c>
       <c r="M22" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N22" t="s">
         <v>3</v>
       </c>
       <c r="O22" s="2">
         <f>O20-O21</f>
-        <v>-14.280000000000001</v>
+        <v>-11.379999999999995</v>
       </c>
       <c r="P22" t="s">
         <v>3</v>
       </c>
       <c r="Q22" s="2">
         <f>Q20-Q21</f>
-        <v>7.5630000000000024</v>
+        <v>6.5762999999999998</v>
       </c>
       <c r="R22" t="s">
         <v>9</v>
       </c>
       <c r="S22" s="2">
         <f>S20-S21</f>
-        <v>5.7204999999999995</v>
+        <v>4.9484999999999992</v>
       </c>
       <c r="T22" t="s">
         <v>9</v>
       </c>
       <c r="U22" s="2">
         <f>U20-U21</f>
-        <v>1.8426000000000009</v>
+        <v>1.6279000000000003</v>
       </c>
       <c r="V22" s="3" t="s">
         <v>4</v>
       </c>
       <c r="X22" s="2" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="Y22" t="s">
         <v>3</v>
       </c>
-      <c r="Z22" s="2">
-        <f>100-Z23</f>
-        <v>77.7</v>
+      <c r="Z22" t="s">
+        <v>10</v>
       </c>
       <c r="AA22" t="s">
         <v>3</v>
       </c>
-      <c r="AB22" s="2">
+      <c r="AB22" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD22" s="2">
+        <f>100-AD23</f>
+        <v>44.31</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF22" s="2">
         <f>Q20</f>
-        <v>28.956800000000001</v>
-      </c>
-      <c r="AC22" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD22" s="2">
+        <v>28.5366</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH22" s="2">
         <f>O26</f>
-        <v>67.86</v>
-      </c>
-      <c r="AE22" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF22" s="2">
+        <v>68.959999999999994</v>
+      </c>
+      <c r="AI22" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ22" s="2">
         <f>Q26</f>
-        <v>30.261800000000001</v>
-      </c>
-      <c r="AG22" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH22" s="2">
-        <f>100-AH23</f>
-        <v>89.5</v>
-      </c>
-      <c r="AI22" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ22" s="2">
+        <v>30.138300000000001</v>
+      </c>
+      <c r="AK22" t="s">
+        <v>9</v>
+      </c>
+      <c r="AL22" s="2">
+        <f>100-AL23</f>
+        <v>93.6</v>
+      </c>
+      <c r="AM22" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN22" s="2">
         <f>Q32</f>
-        <v>33.386800000000001</v>
-      </c>
-      <c r="AK22" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL22" s="2">
-        <f t="shared" ref="AL22:AL24" si="0">AJ22-AB22</f>
-        <v>4.43</v>
-      </c>
-      <c r="AM22" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO22" s="3" t="s">
+        <v>33.424700000000001</v>
+      </c>
+      <c r="AO22" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP22" s="2">
+        <f t="shared" ref="AP22:AP24" si="0">AN22-AF22</f>
+        <v>4.8881000000000014</v>
+      </c>
+      <c r="AQ22" t="s">
+        <v>3</v>
+      </c>
+      <c r="AS22" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="AP22" s="6"/>
-    </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="AT22" s="6"/>
+    </row>
+    <row r="23" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>6</v>
       </c>
@@ -3483,14 +3673,14 @@
       </c>
       <c r="Q23">
         <f>ROUND(Q20*$O20/100+Q21*$O21/100,1)</f>
-        <v>24.6</v>
+        <v>24.9</v>
       </c>
       <c r="R23" t="s">
         <v>9</v>
       </c>
       <c r="S23">
         <f>ROUND(S20*$O20/100+S21*$O21/100,1)</f>
-        <v>14.3</v>
+        <v>14.5</v>
       </c>
       <c r="T23" t="s">
         <v>9</v>
@@ -3503,63 +3693,77 @@
         <v>4</v>
       </c>
       <c r="X23" s="2" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="Y23" t="s">
         <v>3</v>
       </c>
-      <c r="Z23" s="2">
-        <v>22.3</v>
+      <c r="Z23" t="s">
+        <v>10</v>
       </c>
       <c r="AA23" t="s">
         <v>3</v>
       </c>
-      <c r="AB23" s="2">
+      <c r="AB23" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD23" s="2">
+        <f>O21</f>
+        <v>55.69</v>
+      </c>
+      <c r="AE23" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF23" s="2">
         <f>Q21</f>
-        <v>21.393799999999999</v>
-      </c>
-      <c r="AC23" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD23" s="2">
+        <v>21.9603</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH23" s="2">
         <f>O27</f>
-        <v>32.14</v>
-      </c>
-      <c r="AE23" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF23" s="2">
+        <v>31.04</v>
+      </c>
+      <c r="AI23" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ23" s="2">
         <f>Q27</f>
-        <v>23.019400000000001</v>
-      </c>
-      <c r="AG23" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH23" s="2">
-        <v>10.5</v>
-      </c>
-      <c r="AI23" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ23" s="2">
+        <v>23.289100000000001</v>
+      </c>
+      <c r="AK23" t="s">
+        <v>9</v>
+      </c>
+      <c r="AL23" s="2">
+        <f>O33</f>
+        <v>6.4</v>
+      </c>
+      <c r="AM23" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN23" s="2">
         <f>Q33</f>
-        <v>24.4633</v>
-      </c>
-      <c r="AK23" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL23" s="2">
+        <v>23.822600000000001</v>
+      </c>
+      <c r="AO23" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP23" s="2">
         <f t="shared" si="0"/>
-        <v>3.0695000000000014</v>
-      </c>
-      <c r="AM23" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO23" s="3" t="s">
+        <v>1.8623000000000012</v>
+      </c>
+      <c r="AQ23" t="s">
+        <v>3</v>
+      </c>
+      <c r="AS23" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>1</v>
       </c>
@@ -3595,7 +3799,7 @@
         <v>4</v>
       </c>
       <c r="M24" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="N24" t="s">
         <v>3</v>
@@ -3605,85 +3809,97 @@
       </c>
       <c r="Q24">
         <f>ROUND(Q20*$O$32/100+Q21*$O$33/100,1)</f>
-        <v>28.3</v>
+        <v>28.1</v>
       </c>
       <c r="R24" t="s">
         <v>9</v>
       </c>
       <c r="S24" s="2">
         <f>ROUND(S20*$O$32/100+S21*$O$33/100,1)</f>
-        <v>17</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="T24" t="s">
         <v>9</v>
       </c>
       <c r="U24">
         <f>ROUND(U20*$O$32/100+U21*$O$33/100,1)</f>
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="V24" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="X24" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y24" t="s">
         <v>3</v>
       </c>
-      <c r="Z24" s="2">
-        <f>Z22-Z23</f>
-        <v>55.400000000000006</v>
+      <c r="Z24" t="s">
+        <v>10</v>
       </c>
       <c r="AA24" t="s">
         <v>3</v>
       </c>
-      <c r="AB24" s="2">
-        <f>AB22-AB23</f>
-        <v>7.5630000000000024</v>
+      <c r="AB24" t="s">
+        <v>10</v>
       </c>
       <c r="AC24" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD24" s="2">
         <f>AD22-AD23</f>
-        <v>35.72</v>
+        <v>-11.379999999999995</v>
       </c>
       <c r="AE24" t="s">
         <v>3</v>
       </c>
       <c r="AF24" s="2">
         <f>AF22-AF23</f>
-        <v>7.2423999999999999</v>
+        <v>6.5762999999999998</v>
       </c>
       <c r="AG24" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH24" s="2">
         <f>AH22-AH23</f>
-        <v>79</v>
+        <v>37.919999999999995</v>
       </c>
       <c r="AI24" t="s">
         <v>3</v>
       </c>
       <c r="AJ24" s="2">
         <f>AJ22-AJ23</f>
-        <v>8.9235000000000007</v>
-      </c>
-      <c r="AK24" s="3" t="s">
-        <v>3</v>
+        <v>6.8491999999999997</v>
+      </c>
+      <c r="AK24" t="s">
+        <v>9</v>
       </c>
       <c r="AL24" s="2">
+        <f>AL22-AL23</f>
+        <v>87.199999999999989</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN24" s="2">
+        <f>AN22-AN23</f>
+        <v>9.6021000000000001</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP24" s="2">
         <f t="shared" si="0"/>
-        <v>1.3604999999999983</v>
-      </c>
-      <c r="AM24" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO24" s="3" t="s">
+        <v>3.0258000000000003</v>
+      </c>
+      <c r="AQ24" t="s">
+        <v>3</v>
+      </c>
+      <c r="AS24" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>0</v>
       </c>
@@ -3719,7 +3935,7 @@
         <v>4</v>
       </c>
       <c r="M25" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="O25" s="2"/>
       <c r="Q25" s="2"/>
@@ -3729,7 +3945,7 @@
       <c r="AC25" s="2"/>
       <c r="AD25" s="2"/>
     </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>2</v>
       </c>
@@ -3771,28 +3987,28 @@
       </c>
       <c r="O26" s="2">
         <f>M4*100</f>
-        <v>67.86</v>
+        <v>68.959999999999994</v>
       </c>
       <c r="P26" t="s">
         <v>3</v>
       </c>
       <c r="Q26" s="2">
         <f>N4</f>
-        <v>30.261800000000001</v>
+        <v>30.138300000000001</v>
       </c>
       <c r="R26" t="s">
         <v>9</v>
       </c>
       <c r="S26" s="2">
         <f>O4</f>
-        <v>23.8552</v>
+        <v>23.950700000000001</v>
       </c>
       <c r="T26" t="s">
         <v>9</v>
       </c>
       <c r="U26" s="2">
         <f>P4</f>
-        <v>6.4066000000000001</v>
+        <v>6.1875</v>
       </c>
       <c r="V26" s="3" t="s">
         <v>4</v>
@@ -3803,7 +4019,7 @@
       <c r="AC26" s="4"/>
       <c r="AD26" s="4"/>
     </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>7</v>
       </c>
@@ -3820,28 +4036,28 @@
       </c>
       <c r="O27" s="2">
         <f>M5*100</f>
-        <v>32.14</v>
+        <v>31.04</v>
       </c>
       <c r="P27" t="s">
         <v>3</v>
       </c>
       <c r="Q27" s="2">
         <f>N5</f>
-        <v>23.019400000000001</v>
+        <v>23.289100000000001</v>
       </c>
       <c r="R27" t="s">
         <v>9</v>
       </c>
       <c r="S27" s="2">
         <f>O5</f>
-        <v>16.190300000000001</v>
+        <v>16.069099999999999</v>
       </c>
       <c r="T27" t="s">
         <v>9</v>
       </c>
       <c r="U27" s="2">
         <f>P5</f>
-        <v>6.8291000000000004</v>
+        <v>7.2199</v>
       </c>
       <c r="V27" s="3" t="s">
         <v>4</v>
@@ -3852,7 +4068,7 @@
       <c r="AA27" s="2"/>
       <c r="AB27" s="2"/>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -3888,35 +4104,35 @@
         <v>4</v>
       </c>
       <c r="M28" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N28" t="s">
         <v>3</v>
       </c>
       <c r="O28" s="2">
         <f>O26-O27</f>
-        <v>35.72</v>
+        <v>37.919999999999995</v>
       </c>
       <c r="P28" t="s">
         <v>3</v>
       </c>
       <c r="Q28" s="2">
         <f>Q26-Q27</f>
-        <v>7.2423999999999999</v>
+        <v>6.8491999999999997</v>
       </c>
       <c r="R28" t="s">
         <v>9</v>
       </c>
       <c r="S28" s="2">
         <f>S26-S27</f>
-        <v>7.6648999999999994</v>
+        <v>7.8816000000000024</v>
       </c>
       <c r="T28" t="s">
         <v>9</v>
       </c>
       <c r="U28" s="2">
         <f>U26-U27</f>
-        <v>-0.42250000000000032</v>
+        <v>-1.0324</v>
       </c>
       <c r="V28" s="3" t="s">
         <v>4</v>
@@ -3927,7 +4143,7 @@
       <c r="AA28" s="2"/>
       <c r="AB28" s="2"/>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>0</v>
       </c>
@@ -3976,14 +4192,14 @@
       </c>
       <c r="Q29">
         <f>ROUND(Q26*$O26/100+Q27*$O27/100,1)</f>
-        <v>27.9</v>
+        <v>28</v>
       </c>
       <c r="R29" t="s">
         <v>9</v>
       </c>
       <c r="S29">
         <f>ROUND(S26*$O26/100+S27*$O27/100,1)</f>
-        <v>21.4</v>
+        <v>21.5</v>
       </c>
       <c r="T29" t="s">
         <v>9</v>
@@ -3996,7 +4212,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>2</v>
       </c>
@@ -4031,7 +4247,7 @@
         <v>4</v>
       </c>
       <c r="M30" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="N30" t="s">
         <v>3</v>
@@ -4048,20 +4264,20 @@
       </c>
       <c r="S30" s="2">
         <f>ROUND(S26*$O$32/100+S27*$O$33/100,1)</f>
-        <v>23.2</v>
+        <v>23.4</v>
       </c>
       <c r="T30" t="s">
         <v>9</v>
       </c>
       <c r="U30">
         <f>ROUND(U26*$O$32/100+U27*$O$33/100,1)</f>
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="V30" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -4071,7 +4287,7 @@
       <c r="I31" s="2"/>
       <c r="J31" s="3"/>
       <c r="M31" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="O31" s="2"/>
       <c r="Q31" s="2"/>
@@ -4082,31 +4298,31 @@
         <v>3</v>
       </c>
       <c r="Z31" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="AC31" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD31" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="AG31" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH31" t="s">
-        <v>23</v>
-      </c>
-      <c r="AK31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="AK31" t="s">
         <v>3</v>
       </c>
       <c r="AL31" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="AO31" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>1</v>
       </c>
@@ -4149,88 +4365,88 @@
       </c>
       <c r="O32" s="2">
         <f>M6*100</f>
-        <v>91.59</v>
+        <v>93.600000000000009</v>
       </c>
       <c r="P32" t="s">
         <v>3</v>
       </c>
       <c r="Q32" s="2">
         <f>N6</f>
-        <v>33.386800000000001</v>
+        <v>33.424700000000001</v>
       </c>
       <c r="R32" t="s">
         <v>9</v>
       </c>
       <c r="S32" s="2">
         <f>O6</f>
-        <v>29.600899999999999</v>
+        <v>29.8184</v>
       </c>
       <c r="T32" t="s">
         <v>9</v>
       </c>
       <c r="U32" s="2">
         <f>P6</f>
-        <v>3.7858999999999998</v>
+        <v>3.6063000000000001</v>
       </c>
       <c r="V32" s="3" t="s">
         <v>4</v>
       </c>
       <c r="X32" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="Y32" t="s">
         <v>3</v>
       </c>
       <c r="Z32" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AA32" t="s">
         <v>3</v>
       </c>
       <c r="AB32" t="s">
+        <v>23</v>
+      </c>
+      <c r="AC32" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD32" t="s">
+        <v>22</v>
+      </c>
+      <c r="AE32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF32" t="s">
+        <v>23</v>
+      </c>
+      <c r="AG32" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH32" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ32" t="s">
+        <v>23</v>
+      </c>
+      <c r="AK32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL32" t="s">
+        <v>23</v>
+      </c>
+      <c r="AM32" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN32" t="s">
         <v>26</v>
-      </c>
-      <c r="AC32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD32" t="s">
-        <v>25</v>
-      </c>
-      <c r="AE32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF32" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH32" t="s">
-        <v>25</v>
-      </c>
-      <c r="AI32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ32" t="s">
-        <v>26</v>
-      </c>
-      <c r="AK32" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL32" t="s">
-        <v>26</v>
-      </c>
-      <c r="AM32" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN32" t="s">
-        <v>29</v>
       </c>
       <c r="AO32" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>0</v>
       </c>
@@ -4273,34 +4489,34 @@
       </c>
       <c r="O33" s="2">
         <f>M7*100</f>
-        <v>8.41</v>
+        <v>6.4</v>
       </c>
       <c r="P33" t="s">
         <v>3</v>
       </c>
       <c r="Q33" s="2">
         <f>N7</f>
-        <v>24.4633</v>
+        <v>23.822600000000001</v>
       </c>
       <c r="R33" t="s">
         <v>9</v>
       </c>
       <c r="S33" s="2">
         <f>O7</f>
-        <v>19.1035</v>
+        <v>17.418600000000001</v>
       </c>
       <c r="T33" t="s">
         <v>9</v>
       </c>
       <c r="U33" s="2">
         <f>P7</f>
-        <v>5.3597999999999999</v>
+        <v>6.4039999999999999</v>
       </c>
       <c r="V33" s="3" t="s">
         <v>4</v>
       </c>
       <c r="X33" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="Y33" t="s">
         <v>3</v>
@@ -4313,10 +4529,10 @@
       </c>
       <c r="AB33" s="2">
         <f>Z34/100*AB34+Z35/100*AB35</f>
-        <v>27.159746639999998</v>
+        <v>27.230447039999998</v>
       </c>
       <c r="AC33" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD33">
         <v>100</v>
@@ -4326,10 +4542,10 @@
       </c>
       <c r="AF33" s="2">
         <f>AD34/100*AF34+AD35/100*AF35</f>
-        <v>31.19696768</v>
+        <v>31.207702140000002</v>
       </c>
       <c r="AG33" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH33">
         <v>100</v>
@@ -4339,27 +4555,31 @@
       </c>
       <c r="AJ33" s="2">
         <f>AH34/100*AJ34+AH35/100*AJ35</f>
-        <v>34.45117381</v>
-      </c>
-      <c r="AK33" s="3" t="s">
+        <v>34.498373459999996</v>
+      </c>
+      <c r="AK33" t="s">
         <v>3</v>
       </c>
       <c r="AL33" s="2">
         <f>AJ33-AB33</f>
-        <v>7.2914271700000022</v>
+        <v>7.2679264199999984</v>
       </c>
       <c r="AM33" t="s">
         <v>3</v>
       </c>
       <c r="AN33" s="2">
         <f>AJ33-(AB34*AH34/100+AB35*AH35/100)</f>
-        <v>4.6366477999999987</v>
+        <v>4.8576423299999973</v>
       </c>
       <c r="AO33" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="34" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AP33" s="7">
+        <f>(AL33-AN33)/AL33</f>
+        <v>0.33163297902512362</v>
+      </c>
+    </row>
+    <row r="34" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>2</v>
       </c>
@@ -4394,35 +4614,35 @@
         <v>4</v>
       </c>
       <c r="M34" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N34" t="s">
         <v>3</v>
       </c>
       <c r="O34" s="2">
         <f>O32-O33</f>
-        <v>83.18</v>
+        <v>87.2</v>
       </c>
       <c r="P34" t="s">
         <v>3</v>
       </c>
       <c r="Q34" s="2">
         <f>Q32-Q33</f>
-        <v>8.9235000000000007</v>
+        <v>9.6021000000000001</v>
       </c>
       <c r="R34" t="s">
         <v>9</v>
       </c>
       <c r="S34" s="2">
         <f>S32-S33</f>
-        <v>10.497399999999999</v>
+        <v>12.399799999999999</v>
       </c>
       <c r="T34" t="s">
         <v>9</v>
       </c>
       <c r="U34" s="2">
         <f>U32-U33</f>
-        <v>-1.5739000000000001</v>
+        <v>-2.7976999999999999</v>
       </c>
       <c r="V34" s="3" t="s">
         <v>4</v>
@@ -4435,49 +4655,49 @@
       </c>
       <c r="Z34" s="2">
         <f>O38</f>
-        <v>55.44</v>
+        <v>54.879999999999995</v>
       </c>
       <c r="AA34" t="s">
         <v>3</v>
       </c>
       <c r="AB34" s="2">
         <f>Q38</f>
-        <v>30.3338</v>
+        <v>30.038399999999999</v>
       </c>
       <c r="AC34" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD34" s="2">
         <f>O44</f>
-        <v>71.78</v>
+        <v>72.42</v>
       </c>
       <c r="AE34" t="s">
         <v>3</v>
       </c>
       <c r="AF34" s="2">
         <f>Q44</f>
-        <v>33.219099999999997</v>
+        <v>33.209099999999999</v>
       </c>
       <c r="AG34" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH34" s="2">
         <f>O50</f>
-        <v>92.710000000000008</v>
+        <v>93.61</v>
       </c>
       <c r="AI34" t="s">
         <v>3</v>
       </c>
       <c r="AJ34" s="2">
         <f>Q50</f>
-        <v>34.942599999999999</v>
-      </c>
-      <c r="AK34" s="3" t="s">
+        <v>34.973700000000001</v>
+      </c>
+      <c r="AK34" t="s">
         <v>3</v>
       </c>
       <c r="AL34" s="2">
         <f t="shared" ref="AL34:AL35" si="1">AJ34-AB34</f>
-        <v>4.6087999999999987</v>
+        <v>4.9353000000000016</v>
       </c>
       <c r="AM34" t="s">
         <v>3</v>
@@ -4486,7 +4706,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>8</v>
       </c>
@@ -4509,21 +4729,21 @@
       </c>
       <c r="Q35">
         <f>ROUND(Q32*$O32/100+Q33*$O33/100,1)</f>
-        <v>32.6</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="R35" t="s">
         <v>9</v>
       </c>
       <c r="S35">
         <f>ROUND(S32*$O32/100+S33*$O33/100,1)</f>
-        <v>28.7</v>
+        <v>29</v>
       </c>
       <c r="T35" t="s">
         <v>9</v>
       </c>
       <c r="U35">
         <f>ROUND(U32*$O32/100+U33*$O33/100,1)</f>
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="V35" s="3" t="s">
         <v>4</v>
@@ -4536,49 +4756,49 @@
       </c>
       <c r="Z35" s="2">
         <f>O39</f>
-        <v>44.56</v>
+        <v>45.12</v>
       </c>
       <c r="AA35" t="s">
         <v>3</v>
       </c>
       <c r="AB35" s="2">
         <f>Q39</f>
-        <v>23.210699999999999</v>
+        <v>23.815100000000001</v>
       </c>
       <c r="AC35" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD35" s="2">
         <f>O45</f>
-        <v>28.22</v>
+        <v>27.58</v>
       </c>
       <c r="AE35" t="s">
         <v>3</v>
       </c>
       <c r="AF35" s="2">
         <f>Q45</f>
-        <v>26.0535</v>
+        <v>25.952400000000001</v>
       </c>
       <c r="AG35" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH35" s="2">
         <f>O51</f>
-        <v>7.2900000000000009</v>
+        <v>6.39</v>
       </c>
       <c r="AI35" t="s">
         <v>3</v>
       </c>
       <c r="AJ35" s="2">
         <f>Q51</f>
-        <v>28.201499999999999</v>
-      </c>
-      <c r="AK35" s="3" t="s">
+        <v>27.5351</v>
+      </c>
+      <c r="AK35" t="s">
         <v>3</v>
       </c>
       <c r="AL35" s="2">
         <f t="shared" si="1"/>
-        <v>4.9908000000000001</v>
+        <v>3.7199999999999989</v>
       </c>
       <c r="AM35" t="s">
         <v>3</v>
@@ -4587,7 +4807,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>1</v>
       </c>
@@ -4623,7 +4843,7 @@
         <v>4</v>
       </c>
       <c r="M36" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="N36" t="s">
         <v>3</v>
@@ -4633,76 +4853,76 @@
       </c>
       <c r="Q36">
         <f>ROUND(Q32*$O$32/100+Q33*$O$33/100,1)</f>
-        <v>32.6</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="R36" t="s">
         <v>9</v>
       </c>
       <c r="S36" s="2">
         <f>ROUND(S32*$O$32/100+S33*$O$33/100,1)</f>
-        <v>28.7</v>
+        <v>29</v>
       </c>
       <c r="T36" t="s">
         <v>9</v>
       </c>
       <c r="U36">
         <f>ROUND(U32*$O$32/100+U33*$O$33/100,1)</f>
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="V36" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="X36" s="2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="Y36" t="s">
         <v>3</v>
       </c>
       <c r="Z36" s="2">
         <f>Z34-Z35</f>
-        <v>10.879999999999995</v>
+        <v>9.759999999999998</v>
       </c>
       <c r="AA36" t="s">
         <v>3</v>
       </c>
       <c r="AB36" s="2">
         <f>AB34-AB35</f>
-        <v>7.1231000000000009</v>
+        <v>6.2232999999999983</v>
       </c>
       <c r="AC36" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AD36" s="2">
         <f>AD34-AD35</f>
-        <v>43.56</v>
+        <v>44.84</v>
       </c>
       <c r="AE36" t="s">
         <v>3</v>
       </c>
       <c r="AF36" s="2">
         <f>AF34-AF35</f>
-        <v>7.1655999999999977</v>
+        <v>7.2566999999999986</v>
       </c>
       <c r="AG36" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="AH36" s="2">
         <f>AH34-AH35</f>
-        <v>85.42</v>
+        <v>87.22</v>
       </c>
       <c r="AI36" t="s">
         <v>3</v>
       </c>
       <c r="AJ36" s="2">
         <f>AJ34-AJ35</f>
-        <v>6.7410999999999994</v>
-      </c>
-      <c r="AK36" s="3" t="s">
+        <v>7.438600000000001</v>
+      </c>
+      <c r="AK36" t="s">
         <v>3</v>
       </c>
       <c r="AL36" s="2">
         <f>AJ36-AB36</f>
-        <v>-0.38200000000000145</v>
+        <v>1.2153000000000027</v>
       </c>
       <c r="AM36" t="s">
         <v>3</v>
@@ -4711,7 +4931,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>0</v>
       </c>
@@ -4747,7 +4967,7 @@
         <v>4</v>
       </c>
       <c r="M37" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="O37" s="2"/>
       <c r="Q37" s="2"/>
@@ -4760,7 +4980,7 @@
       <c r="AA37" s="2"/>
       <c r="AB37" s="2"/>
     </row>
-    <row r="38" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -4802,28 +5022,28 @@
       </c>
       <c r="O38" s="2">
         <f>M8*100</f>
-        <v>55.44</v>
+        <v>54.879999999999995</v>
       </c>
       <c r="P38" t="s">
         <v>3</v>
       </c>
       <c r="Q38" s="2">
         <f>N8</f>
-        <v>30.3338</v>
+        <v>30.038399999999999</v>
       </c>
       <c r="R38" t="s">
         <v>9</v>
       </c>
       <c r="S38" s="2">
         <f>O8</f>
-        <v>15.0909</v>
+        <v>15.1334</v>
       </c>
       <c r="T38" t="s">
         <v>9</v>
       </c>
       <c r="U38" s="2">
         <f>P8</f>
-        <v>15.242900000000001</v>
+        <v>14.904999999999999</v>
       </c>
       <c r="V38" s="3" t="s">
         <v>4</v>
@@ -4832,9 +5052,20 @@
       <c r="Y38" s="2"/>
       <c r="Z38" s="2"/>
       <c r="AA38" s="2"/>
-      <c r="AB38" s="2"/>
-    </row>
-    <row r="39" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AB38" s="2">
+        <f>AB33-AF21</f>
+        <v>2.3561885099999991</v>
+      </c>
+      <c r="AF38" s="2">
+        <f>AF33-AJ21</f>
+        <v>3.1953938199999996</v>
+      </c>
+      <c r="AJ38" s="2">
+        <f>AJ33-AN21</f>
+        <v>1.6882078599999986</v>
+      </c>
+    </row>
+    <row r="39" spans="1:42" x14ac:dyDescent="0.25">
       <c r="L39" s="2"/>
       <c r="M39" t="s">
         <v>1</v>
@@ -4844,71 +5075,81 @@
       </c>
       <c r="O39" s="2">
         <f>M9*100</f>
-        <v>44.56</v>
+        <v>45.12</v>
       </c>
       <c r="P39" t="s">
         <v>3</v>
       </c>
       <c r="Q39" s="2">
         <f>N9</f>
-        <v>23.210699999999999</v>
+        <v>23.815100000000001</v>
       </c>
       <c r="R39" t="s">
         <v>9</v>
       </c>
       <c r="S39" s="2">
         <f>O9</f>
-        <v>9.9444999999999997</v>
+        <v>10.379899999999999</v>
       </c>
       <c r="T39" t="s">
         <v>9</v>
       </c>
       <c r="U39" s="2">
         <f>P9</f>
-        <v>13.2662</v>
+        <v>13.4352</v>
       </c>
       <c r="V39" s="3" t="s">
         <v>4</v>
       </c>
       <c r="X39" s="2"/>
-    </row>
-    <row r="40" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AB39">
+        <f>AF22*Z34/100+AF23*Z35/100</f>
+        <v>25.569373439999996</v>
+      </c>
+      <c r="AF39" s="2"/>
+      <c r="AJ39" s="2"/>
+    </row>
+    <row r="40" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M40" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N40" t="s">
         <v>3</v>
       </c>
       <c r="O40" s="2">
         <f>O38-O39</f>
-        <v>10.879999999999995</v>
+        <v>9.759999999999998</v>
       </c>
       <c r="P40" t="s">
         <v>3</v>
       </c>
       <c r="Q40" s="2">
         <f>Q38-Q39</f>
-        <v>7.1231000000000009</v>
+        <v>6.2232999999999983</v>
       </c>
       <c r="R40" t="s">
         <v>9</v>
       </c>
       <c r="S40" s="2">
         <f>S38-S39</f>
-        <v>5.1463999999999999</v>
+        <v>4.7535000000000007</v>
       </c>
       <c r="T40" t="s">
         <v>9</v>
       </c>
       <c r="U40" s="2">
         <f>U38-U39</f>
-        <v>1.976700000000001</v>
+        <v>1.4697999999999993</v>
       </c>
       <c r="V40" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="41" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="AB40" s="2">
+        <f>AB33-AB39</f>
+        <v>1.6610736000000017</v>
+      </c>
+    </row>
+    <row r="41" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M41" t="s">
         <v>2</v>
       </c>
@@ -4930,22 +5171,22 @@
       </c>
       <c r="S41">
         <f>ROUND(S38*$O38/100+S39*$O39/100,1)</f>
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="T41" t="s">
         <v>9</v>
       </c>
       <c r="U41">
         <f>ROUND(U38*$O38/100+U39*$O39/100,1)</f>
-        <v>14.4</v>
+        <v>14.2</v>
       </c>
       <c r="V41" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M42" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="N42" t="s">
         <v>3</v>
@@ -4955,29 +5196,29 @@
       </c>
       <c r="Q42">
         <f>ROUND(Q38*$O$50/100+Q39*$O$51/100,1)</f>
-        <v>29.8</v>
+        <v>29.6</v>
       </c>
       <c r="R42" t="s">
         <v>9</v>
       </c>
       <c r="S42">
         <f>ROUND(S38*$O$50/100+S39*$O$51/100,1)</f>
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="T42" t="s">
         <v>9</v>
       </c>
       <c r="U42">
         <f>ROUND(U38*$O$50/100+U39*$O$51/100,1)</f>
-        <v>15.1</v>
+        <v>14.8</v>
       </c>
       <c r="V42" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="43" spans="1:41" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M43" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="O43" s="2"/>
       <c r="Q43" s="2"/>
@@ -4985,7 +5226,7 @@
       <c r="U43" s="2"/>
       <c r="V43" s="3"/>
     </row>
-    <row r="44" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M44" t="s">
         <v>0</v>
       </c>
@@ -4994,34 +5235,34 @@
       </c>
       <c r="O44" s="2">
         <f>M10*100</f>
-        <v>71.78</v>
+        <v>72.42</v>
       </c>
       <c r="P44" t="s">
         <v>3</v>
       </c>
       <c r="Q44" s="2">
         <f>N10</f>
-        <v>33.219099999999997</v>
+        <v>33.209099999999999</v>
       </c>
       <c r="R44" t="s">
         <v>9</v>
       </c>
       <c r="S44" s="2">
         <f>O10</f>
-        <v>25.819900000000001</v>
+        <v>26.057200000000002</v>
       </c>
       <c r="T44" t="s">
         <v>9</v>
       </c>
       <c r="U44" s="2">
         <f>P10</f>
-        <v>7.3992000000000004</v>
+        <v>7.1519000000000004</v>
       </c>
       <c r="V44" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M45" t="s">
         <v>1</v>
       </c>
@@ -5030,73 +5271,73 @@
       </c>
       <c r="O45" s="2">
         <f>M11*100</f>
-        <v>28.22</v>
+        <v>27.58</v>
       </c>
       <c r="P45" t="s">
         <v>3</v>
       </c>
       <c r="Q45" s="2">
         <f>N11</f>
-        <v>26.0535</v>
+        <v>25.952400000000001</v>
       </c>
       <c r="R45" t="s">
         <v>9</v>
       </c>
       <c r="S45" s="2">
         <f>O11</f>
-        <v>17.647300000000001</v>
+        <v>16.8109</v>
       </c>
       <c r="T45" t="s">
         <v>9</v>
       </c>
       <c r="U45" s="2">
         <f>P11</f>
-        <v>8.4062000000000001</v>
+        <v>9.1415000000000006</v>
       </c>
       <c r="V45" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M46" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N46" t="s">
         <v>3</v>
       </c>
       <c r="O46" s="2">
         <f>O44-O45</f>
-        <v>43.56</v>
+        <v>44.84</v>
       </c>
       <c r="P46" t="s">
         <v>3</v>
       </c>
       <c r="Q46" s="2">
         <f>Q44-Q45</f>
-        <v>7.1655999999999977</v>
+        <v>7.2566999999999986</v>
       </c>
       <c r="R46" t="s">
         <v>9</v>
       </c>
       <c r="S46" s="2">
         <f>S44-S45</f>
-        <v>8.1725999999999992</v>
+        <v>9.2463000000000015</v>
       </c>
       <c r="T46" t="s">
         <v>9</v>
       </c>
       <c r="U46" s="2">
         <f>U44-U45</f>
-        <v>-1.0069999999999997</v>
+        <v>-1.9896000000000003</v>
       </c>
       <c r="V46" s="3" t="s">
         <v>4</v>
       </c>
       <c r="AD46" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="47" spans="1:41" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="47" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M47" t="s">
         <v>2</v>
       </c>
@@ -5138,9 +5379,9 @@
         <v>0.22325993522498114</v>
       </c>
     </row>
-    <row r="48" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:42" x14ac:dyDescent="0.25">
       <c r="M48" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="N48" t="s">
         <v>3</v>
@@ -5157,17 +5398,17 @@
       </c>
       <c r="S48">
         <f>ROUND(S44*$O$50/100+S45*$O$51/100,1)</f>
-        <v>25.2</v>
+        <v>25.5</v>
       </c>
       <c r="T48" t="s">
         <v>9</v>
       </c>
       <c r="U48">
         <f>ROUND(U44*$O$50/100+U45*$O$51/100,1)</f>
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="V48" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="AD48">
         <v>0.30206</v>
@@ -5175,7 +5416,7 @@
     </row>
     <row r="49" spans="7:30" x14ac:dyDescent="0.25">
       <c r="M49" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="O49" s="2"/>
       <c r="Q49" s="2"/>
@@ -5184,7 +5425,7 @@
       <c r="V49" s="3"/>
       <c r="X49" s="5">
         <f>(X38-Q40)/(Q52-Q40)</f>
-        <v>18.646858638743389</v>
+        <v>-5.1207932197811115</v>
       </c>
       <c r="Y49" s="5"/>
       <c r="Z49" s="5"/>
@@ -5201,28 +5442,28 @@
       </c>
       <c r="O50" s="2">
         <f>M12*100</f>
-        <v>92.710000000000008</v>
+        <v>93.61</v>
       </c>
       <c r="P50" t="s">
         <v>3</v>
       </c>
       <c r="Q50" s="2">
         <f>N12</f>
-        <v>34.942599999999999</v>
+        <v>34.973700000000001</v>
       </c>
       <c r="R50" t="s">
         <v>9</v>
       </c>
       <c r="S50" s="2">
         <f>O12</f>
-        <v>30.402899999999999</v>
+        <v>30.670500000000001</v>
       </c>
       <c r="T50" t="s">
         <v>9</v>
       </c>
       <c r="U50" s="2">
         <f>P12</f>
-        <v>4.5396999999999998</v>
+        <v>4.3032000000000004</v>
       </c>
       <c r="V50" s="3" t="s">
         <v>4</v>
@@ -5240,28 +5481,28 @@
       </c>
       <c r="O51" s="2">
         <f>M13*100</f>
-        <v>7.2900000000000009</v>
+        <v>6.39</v>
       </c>
       <c r="P51" t="s">
         <v>3</v>
       </c>
       <c r="Q51" s="2">
         <f>N13</f>
-        <v>28.201499999999999</v>
+        <v>27.5351</v>
       </c>
       <c r="R51" t="s">
         <v>9</v>
       </c>
       <c r="S51" s="2">
         <f>O13</f>
-        <v>20.847899999999999</v>
+        <v>18.8123</v>
       </c>
       <c r="T51" t="s">
         <v>9</v>
       </c>
       <c r="U51" s="2">
         <f>P13</f>
-        <v>7.3536000000000001</v>
+        <v>8.7227999999999994</v>
       </c>
       <c r="V51" s="3" t="s">
         <v>4</v>
@@ -5272,35 +5513,35 @@
     </row>
     <row r="52" spans="7:30" x14ac:dyDescent="0.25">
       <c r="M52" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="N52" t="s">
         <v>3</v>
       </c>
       <c r="O52" s="2">
         <f>O50-O51</f>
-        <v>85.42</v>
+        <v>87.22</v>
       </c>
       <c r="P52" t="s">
         <v>3</v>
       </c>
       <c r="Q52" s="2">
         <f>Q50-Q51</f>
-        <v>6.7410999999999994</v>
+        <v>7.438600000000001</v>
       </c>
       <c r="R52" t="s">
         <v>9</v>
       </c>
       <c r="S52" s="2">
         <f>S50-S51</f>
-        <v>9.5549999999999997</v>
+        <v>11.8582</v>
       </c>
       <c r="T52" t="s">
         <v>9</v>
       </c>
       <c r="U52" s="2">
         <f>U50-U51</f>
-        <v>-2.8139000000000003</v>
+        <v>-4.4195999999999991</v>
       </c>
       <c r="V52" s="3" t="s">
         <v>4</v>
@@ -5331,14 +5572,14 @@
       </c>
       <c r="S53">
         <f>ROUND(S50*$O50/100+S51*$O51/100,1)</f>
-        <v>29.7</v>
+        <v>29.9</v>
       </c>
       <c r="T53" t="s">
         <v>9</v>
       </c>
       <c r="U53">
         <f>ROUND(U50*$O50/100+U51*$O51/100,1)</f>
-        <v>4.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="V53" s="3" t="s">
         <v>4</v>
@@ -5347,7 +5588,7 @@
     <row r="54" spans="7:30" x14ac:dyDescent="0.25">
       <c r="L54" s="2"/>
       <c r="M54" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="N54" t="s">
         <v>3</v>
@@ -5364,22 +5605,22 @@
       </c>
       <c r="S54">
         <f>ROUND(S50*$O$50/100+S51*$O$51/100,1)</f>
-        <v>29.7</v>
+        <v>29.9</v>
       </c>
       <c r="T54" t="s">
         <v>9</v>
       </c>
       <c r="U54">
         <f>ROUND(U50*$O$50/100+U51*$O$51/100,1)</f>
-        <v>4.7</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="V54" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="62" spans="7:30" x14ac:dyDescent="0.25">
       <c r="G62" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H62">
         <v>0.31209999999999999</v>
@@ -5396,7 +5637,7 @@
     </row>
     <row r="63" spans="7:30" x14ac:dyDescent="0.25">
       <c r="G63" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H63">
         <v>0.35170000000000001</v>
@@ -5413,7 +5654,7 @@
     </row>
     <row r="64" spans="7:30" x14ac:dyDescent="0.25">
       <c r="G64" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H64">
         <v>0.33629999999999999</v>
@@ -5691,12 +5932,12 @@
     <hyperlink ref="V52" r:id="rId34" xr:uid="{E08D1C24-C16D-46DC-BB86-F7E28EA8C801}"/>
     <hyperlink ref="V51" r:id="rId35" xr:uid="{4AEFECD8-657C-4782-9168-4AC29C93DB61}"/>
     <hyperlink ref="V20" r:id="rId36" xr:uid="{59E4A939-1BAA-4206-9E1F-F7D7D5A9D415}"/>
-    <hyperlink ref="AO19" r:id="rId37" xr:uid="{388742D3-27AA-48B1-B26C-58EEEAEF80F6}"/>
-    <hyperlink ref="AO20" r:id="rId38" xr:uid="{5B769362-DA01-4CC7-9250-05B69E2F6891}"/>
-    <hyperlink ref="AO21" r:id="rId39" xr:uid="{C6E61F4E-9248-4F3A-B1DF-1DEFAC22C418}"/>
-    <hyperlink ref="AO22" r:id="rId40" xr:uid="{BE109620-8BE6-4D10-B132-A344C7881E3F}"/>
-    <hyperlink ref="AO23" r:id="rId41" xr:uid="{DA8F37C1-8F15-473A-A5D2-D87FC52B8278}"/>
-    <hyperlink ref="AO24" r:id="rId42" xr:uid="{B04D7A7B-4841-465F-82AE-83966B7B9BEC}"/>
+    <hyperlink ref="AS19" r:id="rId37" xr:uid="{388742D3-27AA-48B1-B26C-58EEEAEF80F6}"/>
+    <hyperlink ref="AS20" r:id="rId38" xr:uid="{5B769362-DA01-4CC7-9250-05B69E2F6891}"/>
+    <hyperlink ref="AS21" r:id="rId39" xr:uid="{C6E61F4E-9248-4F3A-B1DF-1DEFAC22C418}"/>
+    <hyperlink ref="AS22" r:id="rId40" xr:uid="{BE109620-8BE6-4D10-B132-A344C7881E3F}"/>
+    <hyperlink ref="AS23" r:id="rId41" xr:uid="{DA8F37C1-8F15-473A-A5D2-D87FC52B8278}"/>
+    <hyperlink ref="AS24" r:id="rId42" xr:uid="{B04D7A7B-4841-465F-82AE-83966B7B9BEC}"/>
     <hyperlink ref="AO31" r:id="rId43" xr:uid="{B283F196-AD07-4D61-8724-8C370E36802B}"/>
     <hyperlink ref="AO32" r:id="rId44" xr:uid="{DBCA8C43-33A9-44A6-BB2D-EA3515B0AB86}"/>
     <hyperlink ref="AO33" r:id="rId45" xr:uid="{321DA888-BB9B-4B0C-A83F-19101D8E2306}"/>
@@ -5707,697 +5948,390 @@
     <hyperlink ref="V23" r:id="rId50" xr:uid="{532914B8-8922-43FC-BD51-370E140EA6FF}"/>
     <hyperlink ref="V29" r:id="rId51" xr:uid="{09C4ED3A-6F4A-4BBB-BF61-BB03834793D9}"/>
     <hyperlink ref="V35" r:id="rId52" xr:uid="{0BB8DAE4-5467-4575-B09D-7653BA53B50E}"/>
-    <hyperlink ref="V54" r:id="rId53" xr:uid="{2FE7D5EC-94ED-4BAC-BF9D-B76FF3451E99}"/>
-    <hyperlink ref="V47" r:id="rId54" xr:uid="{50ABAC46-1965-4A8E-A051-77034556F45A}"/>
-    <hyperlink ref="V41" r:id="rId55" xr:uid="{41CB5E74-45F6-442A-82C4-D6148AA6031E}"/>
+    <hyperlink ref="V47" r:id="rId53" xr:uid="{50ABAC46-1965-4A8E-A051-77034556F45A}"/>
+    <hyperlink ref="V41" r:id="rId54" xr:uid="{41CB5E74-45F6-442A-82C4-D6148AA6031E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId56"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId55"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A2197B-3151-4F46-B995-07E5FBB54E6A}">
-  <dimension ref="D3:O47"/>
+  <dimension ref="G3:Q47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E3">
-        <v>0.26519999999999999</v>
-      </c>
-      <c r="F3">
-        <v>24.934000000000001</v>
-      </c>
-      <c r="G3">
-        <v>13.7661</v>
-      </c>
-      <c r="H3">
-        <v>11.167899999999999</v>
-      </c>
-      <c r="J3" s="2">
-        <f>E3*F3</f>
-        <v>6.6124967999999997</v>
-      </c>
-      <c r="K3" s="2">
-        <f>F3*E19</f>
-        <v>12.793635400000001</v>
-      </c>
-      <c r="N3" s="2">
-        <f>F3*E27</f>
-        <v>6.4105314</v>
-      </c>
-    </row>
-    <row r="4" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E4">
-        <v>0.1145</v>
-      </c>
-      <c r="F4">
-        <v>21.952400000000001</v>
-      </c>
-      <c r="G4">
-        <v>9.9632000000000005</v>
-      </c>
-      <c r="H4">
-        <v>11.9892</v>
-      </c>
-      <c r="J4" s="2">
-        <f>E4*F4</f>
-        <v>2.5135498000000003</v>
-      </c>
-      <c r="K4" s="2">
-        <f>F4*E20</f>
-        <v>2.3884211199999998</v>
-      </c>
-      <c r="N4" s="2">
-        <f>F4*E28</f>
-        <v>4.4168228799999998</v>
-      </c>
-    </row>
-    <row r="5" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E5">
-        <v>0.32819999999999999</v>
-      </c>
-      <c r="F5">
-        <v>25.076499999999999</v>
-      </c>
-      <c r="G5">
-        <v>14.881</v>
-      </c>
-      <c r="H5">
-        <v>10.195499999999999</v>
-      </c>
-      <c r="J5" s="2">
-        <f>E5*F5</f>
-        <v>8.2301073000000002</v>
-      </c>
-      <c r="K5" s="2">
-        <f>F5*E21</f>
-        <v>6.9913281999999999</v>
-      </c>
-      <c r="N5" s="2">
-        <f>F5*E29</f>
-        <v>8.1147554</v>
-      </c>
-    </row>
-    <row r="6" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E6">
-        <v>0.29210000000000003</v>
-      </c>
-      <c r="F6">
-        <v>17.442</v>
-      </c>
-      <c r="G6">
-        <v>8.4137000000000004</v>
-      </c>
-      <c r="H6">
-        <v>9.0282999999999998</v>
-      </c>
-      <c r="J6" s="2">
-        <f>E6*F6</f>
-        <v>5.0948082000000001</v>
-      </c>
-      <c r="K6" s="2">
-        <f>F6*E22</f>
-        <v>1.7302464</v>
-      </c>
-      <c r="L6" t="s">
-        <v>15</v>
-      </c>
-      <c r="N6" s="2">
-        <f>F6*E30</f>
-        <v>3.8041001999999997</v>
+    <row r="3" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="L3" s="2"/>
+    </row>
+    <row r="4" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="L4" s="2"/>
+    </row>
+    <row r="5" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="O6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J7" s="2">
-        <f>SUM(J3:J6)</f>
-        <v>22.450962100000002</v>
-      </c>
-      <c r="K7" s="2">
-        <f>SUM(K3:K6)</f>
-        <v>23.90363112</v>
-      </c>
-      <c r="L7" s="6">
-        <f>(K7-J7)/(J23-J7)</f>
-        <v>0.1962410673438717</v>
-      </c>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="2">
+        <v>28.5366</v>
+      </c>
+      <c r="I7" s="2">
+        <v>33.424700000000001</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="4">
+        <v>0.68</v>
+      </c>
+      <c r="L7" s="4">
+        <v>0.88</v>
+      </c>
+      <c r="M7" s="6"/>
       <c r="N7" s="2">
-        <f>SUM(N3:N6)</f>
-        <v>22.746209880000002</v>
-      </c>
-      <c r="O7" s="6">
-        <f>(N7-J7)/(J31-J7)</f>
-        <v>8.6000493514011261E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J8" s="2"/>
-    </row>
-    <row r="9" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E11">
-        <v>0.34420000000000001</v>
-      </c>
-      <c r="F11">
-        <v>28.527000000000001</v>
-      </c>
-      <c r="G11">
-        <v>22.930800000000001</v>
-      </c>
-      <c r="H11">
-        <v>5.5961999999999996</v>
-      </c>
-      <c r="J11" s="2">
-        <f>E11*F11</f>
-        <v>9.8189934000000001</v>
-      </c>
-      <c r="N11" s="2">
-        <f>F11*E35</f>
-        <v>10.874492399999999</v>
-      </c>
-    </row>
-    <row r="12" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E12">
-        <v>0.13320000000000001</v>
-      </c>
-      <c r="F12">
-        <v>24.970600000000001</v>
-      </c>
-      <c r="G12">
-        <v>16.799499999999998</v>
+        <f>H7*K7+H8*K8</f>
+        <v>26.432183999999999</v>
+      </c>
+      <c r="O7" s="2">
+        <f>I7*L7+I8*L8</f>
+        <v>32.272447999999997</v>
+      </c>
+      <c r="Q7">
+        <f>O7-N7</f>
+        <v>5.8402639999999977</v>
+      </c>
+    </row>
+    <row r="8" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H8" s="2">
+        <v>21.9603</v>
+      </c>
+      <c r="I8" s="2">
+        <v>23.822600000000001</v>
+      </c>
+      <c r="K8" s="4">
+        <f>1-K7</f>
+        <v>0.31999999999999995</v>
+      </c>
+      <c r="L8" s="4">
+        <f>1-L7</f>
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="9" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="I11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="K11" t="s">
+        <v>55</v>
+      </c>
+      <c r="L11" s="2"/>
+      <c r="M11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G12" s="4">
+        <v>0.44</v>
       </c>
       <c r="H12">
-        <v>8.1710999999999991</v>
+        <v>28.5366</v>
+      </c>
+      <c r="I12" s="2">
+        <f>H12*G12+H13*G13</f>
+        <v>24.853872000000003</v>
       </c>
       <c r="J12" s="2">
-        <f>E12*F12</f>
-        <v>3.3260839200000003</v>
+        <f>I16-I12</f>
+        <v>7.546127999999996</v>
+      </c>
+      <c r="K12" s="2">
+        <f>H16*G12+H17*G13</f>
+        <v>28.047524000000003</v>
+      </c>
+      <c r="L12" s="2">
+        <f>I16-K12</f>
+        <v>4.3524759999999958</v>
+      </c>
+      <c r="M12" s="2">
+        <f>G16*H12+G17*H13</f>
+        <v>27.747443999999998</v>
       </c>
       <c r="N12" s="2">
-        <f>F12*E36</f>
-        <v>4.6844845599999996</v>
-      </c>
-    </row>
-    <row r="13" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E13">
-        <v>0.31040000000000001</v>
-      </c>
-      <c r="F13">
-        <v>27.068100000000001</v>
-      </c>
-      <c r="G13">
-        <v>22.1294</v>
+        <f>I16-M12</f>
+        <v>4.6525560000000006</v>
+      </c>
+    </row>
+    <row r="13" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G13" s="4">
+        <f>1-G12</f>
+        <v>0.56000000000000005</v>
       </c>
       <c r="H13">
-        <v>4.9386999999999999</v>
-      </c>
-      <c r="J13" s="2">
-        <f>E13*F13</f>
-        <v>8.4019382399999998</v>
-      </c>
-      <c r="N13" s="2">
-        <f>F13*E37</f>
-        <v>6.9077791199999998</v>
-      </c>
-    </row>
-    <row r="14" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E14">
-        <v>0.2122</v>
-      </c>
-      <c r="F14">
-        <v>19.4451</v>
-      </c>
-      <c r="G14">
-        <v>13.501899999999999</v>
-      </c>
-      <c r="H14">
-        <v>5.9432</v>
-      </c>
-      <c r="J14" s="2">
-        <f>E14*F14</f>
-        <v>4.1262502200000002</v>
-      </c>
-      <c r="N14" s="2">
-        <f>F14*E38</f>
-        <v>3.4223375999999996</v>
-      </c>
-      <c r="O14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J15" s="2">
-        <f>SUM(J11:J14)</f>
-        <v>25.673265779999998</v>
-      </c>
-      <c r="N15" s="2">
-        <f>SUM(N11:N14)</f>
-        <v>25.889093679999998</v>
-      </c>
-      <c r="O15" s="6">
-        <f>(N15-J15)/(J39-J15)</f>
-        <v>6.1445906540809302E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="D17" t="s">
-        <v>13</v>
-      </c>
-      <c r="E17" t="s">
-        <v>14</v>
-      </c>
-      <c r="J17" s="2"/>
-    </row>
-    <row r="18" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J18" s="2"/>
-    </row>
-    <row r="19" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E19">
-        <v>0.5131</v>
-      </c>
-      <c r="F19">
-        <v>32.189100000000003</v>
-      </c>
-      <c r="G19">
-        <v>28.947099999999999</v>
-      </c>
-      <c r="H19">
-        <v>3.242</v>
-      </c>
-      <c r="J19" s="2">
-        <f>E19*F19</f>
-        <v>16.51622721</v>
-      </c>
-      <c r="N19" s="2">
-        <f>F19*E43</f>
-        <v>16.432535550000001</v>
-      </c>
-    </row>
-    <row r="20" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E20">
-        <v>0.10879999999999999</v>
-      </c>
-      <c r="F20">
-        <v>26.723199999999999</v>
-      </c>
-      <c r="G20">
-        <v>20.771799999999999</v>
-      </c>
-      <c r="H20">
-        <v>5.9513999999999996</v>
-      </c>
-      <c r="J20" s="2">
-        <f>E20*F20</f>
-        <v>2.9074841599999997</v>
-      </c>
-      <c r="N20" s="2">
-        <f>F20*E44</f>
-        <v>4.4066556799999992</v>
-      </c>
-    </row>
-    <row r="21" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E21">
-        <v>0.27879999999999999</v>
-      </c>
-      <c r="F21">
-        <v>29.885400000000001</v>
-      </c>
-      <c r="G21">
-        <v>26.9544</v>
-      </c>
-      <c r="H21">
-        <v>2.931</v>
-      </c>
-      <c r="J21" s="2">
-        <f>E21*F21</f>
-        <v>8.33204952</v>
-      </c>
-      <c r="N21" s="2">
-        <f>F21*E45</f>
-        <v>7.0619200200000005</v>
-      </c>
-    </row>
-    <row r="22" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E22">
-        <v>9.9199999999999997E-2</v>
-      </c>
-      <c r="F22">
-        <v>21.145900000000001</v>
-      </c>
-      <c r="G22">
-        <v>16.101500000000001</v>
-      </c>
-      <c r="H22">
-        <v>5.0445000000000002</v>
-      </c>
-      <c r="J22" s="2">
-        <f>E22*F22</f>
-        <v>2.09767328</v>
-      </c>
-      <c r="N22" s="2">
-        <f>F22*E46</f>
-        <v>1.8671829700000002</v>
-      </c>
-      <c r="O22" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J23" s="2">
-        <f>SUM(J19:J22)</f>
-        <v>29.853434169999996</v>
-      </c>
-      <c r="N23" s="2">
-        <f>SUM(N19:N22)</f>
-        <v>29.768294220000001</v>
-      </c>
-      <c r="O23" s="6">
-        <f>(N23-J23)/(J47-J23)</f>
-        <v>-2.852270811245556E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J24" s="2"/>
-    </row>
-    <row r="25" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25" t="s">
-        <v>14</v>
-      </c>
-      <c r="J25" s="2"/>
-    </row>
-    <row r="26" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J26" s="2"/>
-    </row>
-    <row r="27" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E27">
-        <v>0.2571</v>
-      </c>
-      <c r="F27">
-        <v>28.834399999999999</v>
-      </c>
-      <c r="G27">
-        <v>16.236999999999998</v>
-      </c>
-      <c r="H27">
-        <v>12.5974</v>
-      </c>
-      <c r="J27" s="2">
-        <f>E27*F27</f>
-        <v>7.4133242399999997</v>
-      </c>
-      <c r="K27" s="2">
-        <f>F27*E43</f>
-        <v>14.719961199999998</v>
-      </c>
-    </row>
-    <row r="28" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E28">
-        <v>0.20119999999999999</v>
-      </c>
-      <c r="F28">
-        <v>24.836300000000001</v>
-      </c>
-      <c r="G28">
-        <v>10.030900000000001</v>
-      </c>
-      <c r="H28">
-        <v>14.8055</v>
-      </c>
-      <c r="J28" s="2">
-        <f>E28*F28</f>
-        <v>4.99706356</v>
-      </c>
-      <c r="K28" s="2">
-        <f>F28*E44</f>
-        <v>4.0955058700000002</v>
-      </c>
-    </row>
-    <row r="29" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E29">
-        <v>0.3236</v>
-      </c>
-      <c r="F29">
-        <v>27.988700000000001</v>
-      </c>
-      <c r="G29">
-        <v>16.170200000000001</v>
-      </c>
-      <c r="H29">
-        <v>11.8185</v>
-      </c>
-      <c r="J29" s="2">
-        <f>E29*F29</f>
-        <v>9.0571433199999998</v>
-      </c>
-      <c r="K29" s="2">
-        <f>F29*E45</f>
-        <v>6.6137298100000006</v>
-      </c>
-    </row>
-    <row r="30" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="E30">
-        <v>0.21809999999999999</v>
-      </c>
-      <c r="F30">
-        <v>20.25</v>
-      </c>
-      <c r="G30">
-        <v>9.3089999999999993</v>
-      </c>
-      <c r="H30">
-        <v>10.9411</v>
-      </c>
-      <c r="J30" s="2">
-        <f>E30*F30</f>
-        <v>4.416525</v>
-      </c>
-      <c r="K30" s="2">
-        <f>F30*E46</f>
-        <v>1.7880750000000001</v>
-      </c>
-      <c r="L30" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J31" s="2">
-        <f>SUM(J27:J30)</f>
-        <v>25.884056119999997</v>
-      </c>
-      <c r="K31" s="2">
-        <f>SUM(K27:K30)</f>
-        <v>27.217271879999998</v>
-      </c>
-      <c r="L31" s="4">
-        <f>(K31-J31)/(J47-J31)</f>
-        <v>0.19170916412823169</v>
-      </c>
-    </row>
-    <row r="32" spans="4:15" x14ac:dyDescent="0.25">
-      <c r="J32" s="2"/>
-    </row>
-    <row r="33" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D33" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" t="s">
-        <v>14</v>
-      </c>
-      <c r="J33" s="2"/>
-    </row>
-    <row r="34" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="J34" s="2"/>
-    </row>
-    <row r="35" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E35">
-        <v>0.38119999999999998</v>
-      </c>
-      <c r="F35">
-        <v>32.313499999999998</v>
-      </c>
-      <c r="G35">
-        <v>26.153300000000002</v>
-      </c>
-      <c r="H35">
-        <v>6.1601999999999997</v>
-      </c>
-      <c r="J35" s="2">
-        <f>E35*F35</f>
-        <v>12.317906199999998</v>
-      </c>
-    </row>
-    <row r="36" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E36">
-        <v>0.18759999999999999</v>
-      </c>
-      <c r="F36">
-        <v>27.8371</v>
-      </c>
-      <c r="G36">
-        <v>17.9758</v>
-      </c>
-      <c r="H36">
-        <v>9.8613</v>
-      </c>
-      <c r="J36" s="2">
-        <f>E36*F36</f>
-        <v>5.2222399599999996</v>
-      </c>
-    </row>
-    <row r="37" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E37">
-        <v>0.25519999999999998</v>
-      </c>
-      <c r="F37">
-        <v>30.1967</v>
-      </c>
-      <c r="G37">
-        <v>24.53</v>
-      </c>
-      <c r="H37">
-        <v>5.6666999999999996</v>
-      </c>
-      <c r="J37" s="2">
-        <f>E37*F37</f>
-        <v>7.7061978399999997</v>
-      </c>
-    </row>
-    <row r="38" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E38">
-        <v>0.17599999999999999</v>
-      </c>
-      <c r="F38">
-        <v>22.382999999999999</v>
-      </c>
-      <c r="G38">
-        <v>15.0101</v>
-      </c>
-      <c r="H38">
-        <v>7.3727999999999998</v>
-      </c>
-      <c r="J38" s="2">
-        <f>E38*F38</f>
-        <v>3.9394079999999998</v>
-      </c>
-    </row>
-    <row r="39" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="J39" s="2">
-        <f>SUM(J35:J38)</f>
-        <v>29.185752000000001</v>
-      </c>
-    </row>
-    <row r="40" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="J40" s="2"/>
-    </row>
-    <row r="41" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="D41" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" t="s">
-        <v>14</v>
-      </c>
-      <c r="J41" s="2"/>
-    </row>
-    <row r="42" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="J42" s="2"/>
-    </row>
-    <row r="43" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E43">
-        <v>0.51049999999999995</v>
-      </c>
-      <c r="F43">
-        <v>35.317399999999999</v>
-      </c>
-      <c r="G43">
-        <v>31.659400000000002</v>
-      </c>
-      <c r="H43">
-        <v>3.6579999999999999</v>
-      </c>
-      <c r="J43" s="2">
-        <f>E43*F43</f>
-        <v>18.029532699999997</v>
-      </c>
-    </row>
-    <row r="44" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E44">
-        <v>0.16489999999999999</v>
-      </c>
-      <c r="F44">
-        <v>29.812200000000001</v>
-      </c>
-      <c r="G44">
-        <v>22.9757</v>
-      </c>
-      <c r="H44">
-        <v>6.8365</v>
-      </c>
-      <c r="J44" s="2">
-        <f>E44*F44</f>
-        <v>4.91603178</v>
-      </c>
-    </row>
-    <row r="45" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E45">
-        <v>0.23630000000000001</v>
-      </c>
-      <c r="F45">
-        <v>32.663600000000002</v>
-      </c>
-      <c r="G45">
-        <v>29.0745</v>
-      </c>
-      <c r="H45">
-        <v>3.5891000000000002</v>
-      </c>
-      <c r="J45" s="2">
-        <f>E45*F45</f>
-        <v>7.7184086800000005</v>
-      </c>
-    </row>
-    <row r="46" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="E46">
-        <v>8.8300000000000003E-2</v>
-      </c>
-      <c r="F46">
-        <v>24.625699999999998</v>
-      </c>
-      <c r="G46">
-        <v>18.864100000000001</v>
-      </c>
-      <c r="H46">
-        <v>5.7615999999999996</v>
-      </c>
-      <c r="J46" s="2">
-        <f>E46*F46</f>
-        <v>2.17444931</v>
-      </c>
-    </row>
-    <row r="47" spans="4:10" x14ac:dyDescent="0.25">
-      <c r="J47" s="2">
-        <f>SUM(J43:J46)</f>
-        <v>32.838422469999998</v>
-      </c>
+        <v>21.9603</v>
+      </c>
+      <c r="I13" s="2"/>
+      <c r="L13" s="4">
+        <f>(J12-L12)/J12</f>
+        <v>0.42321731091759929</v>
+      </c>
+      <c r="N13">
+        <f>(J12-N12)/J12</f>
+        <v>0.38345122160663014</v>
+      </c>
+      <c r="P13" s="4">
+        <f>L13+N13</f>
+        <v>0.80666853252422943</v>
+      </c>
+    </row>
+    <row r="14" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G14" s="4"/>
+      <c r="I14" s="2"/>
+      <c r="L14" s="10"/>
+    </row>
+    <row r="15" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G15" s="4"/>
+      <c r="I15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="6"/>
+    </row>
+    <row r="16" spans="7:17" x14ac:dyDescent="0.25">
+      <c r="G16" s="4">
+        <v>0.88</v>
+      </c>
+      <c r="H16">
+        <v>33.424700000000001</v>
+      </c>
+      <c r="I16" s="2">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="17" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="G17" s="4">
+        <f>1-G16</f>
+        <v>0.12</v>
+      </c>
+      <c r="H17">
+        <v>23.822600000000001</v>
+      </c>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I19" s="2"/>
+      <c r="L19" s="2"/>
+    </row>
+    <row r="20" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I20" s="2"/>
+      <c r="L20" s="2"/>
+    </row>
+    <row r="21" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I21" s="2"/>
+      <c r="L21" s="2"/>
+    </row>
+    <row r="22" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I22" s="2"/>
+      <c r="L22" s="2"/>
+    </row>
+    <row r="23" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="G23">
+        <v>0.746</v>
+      </c>
+      <c r="H23">
+        <v>0.71</v>
+      </c>
+      <c r="I23" s="9">
+        <f>G23-H23</f>
+        <v>3.6000000000000032E-2</v>
+      </c>
+      <c r="K23">
+        <v>7.4</v>
+      </c>
+      <c r="L23" s="2"/>
+      <c r="M23" s="6"/>
+    </row>
+    <row r="24" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="G24">
+        <v>0.73499999999999999</v>
+      </c>
+      <c r="H24">
+        <v>0.71199999999999997</v>
+      </c>
+      <c r="I24" s="9">
+        <f>G24-H24</f>
+        <v>2.300000000000002E-2</v>
+      </c>
+      <c r="K24">
+        <v>4.7</v>
+      </c>
+      <c r="L24">
+        <f>K23-K24</f>
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="25" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I25" s="2"/>
+      <c r="K25">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="L25">
+        <f>K23-K25</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I26" s="2"/>
+    </row>
+    <row r="27" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="I30" s="2"/>
+      <c r="J30" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K30" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="H31">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="I31">
+        <v>0.21</v>
+      </c>
+      <c r="J31" s="4">
+        <f>H31+I31</f>
+        <v>0.5</v>
+      </c>
+      <c r="K31" s="4">
+        <f t="shared" ref="K31:K32" si="0">I31/J31</f>
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="32" spans="7:13" x14ac:dyDescent="0.25">
+      <c r="H32">
+        <v>0.19</v>
+      </c>
+      <c r="I32" s="8">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="J32" s="4">
+        <f t="shared" ref="J32:J33" si="1">H32+I32</f>
+        <v>0.255</v>
+      </c>
+      <c r="K32" s="4">
+        <f t="shared" si="0"/>
+        <v>0.25490196078431371</v>
+      </c>
+    </row>
+    <row r="33" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H33">
+        <v>0.2</v>
+      </c>
+      <c r="I33" s="8">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="J33" s="4">
+        <f t="shared" si="1"/>
+        <v>0.22800000000000001</v>
+      </c>
+      <c r="K33" s="4">
+        <f>I33/J33</f>
+        <v>0.12280701754385964</v>
+      </c>
+    </row>
+    <row r="34" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I34" s="2"/>
+    </row>
+    <row r="35" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I35" s="2"/>
+    </row>
+    <row r="36" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I36" s="2"/>
+    </row>
+    <row r="37" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I37" s="2"/>
+    </row>
+    <row r="38" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I38" s="2"/>
+    </row>
+    <row r="39" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I39" s="2"/>
+    </row>
+    <row r="40" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I40" s="2"/>
+    </row>
+    <row r="41" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I41" s="2"/>
+    </row>
+    <row r="42" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I42" s="2"/>
+    </row>
+    <row r="43" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I43" s="2"/>
+    </row>
+    <row r="44" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I44" s="2"/>
+    </row>
+    <row r="45" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I45" s="2"/>
+    </row>
+    <row r="46" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I46" s="2"/>
+    </row>
+    <row r="47" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="I47" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
stated to change habits vars into med and non-med
</commit_message>
<xml_diff>
--- a/Results/table2latex.xlsx
+++ b/Results/table2latex.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbueren\Google Drive\endo_health\metric_model\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71DE7C36-ACEA-43FA-A795-AD3C59EF2988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E69829-7597-442B-9627-478B9D428F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{4D131852-BDAB-48D2-B0B4-24C9607E5D25}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4D131852-BDAB-48D2-B0B4-24C9607E5D25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2536,28 +2536,16 @@
         <v>9.3678000000000008</v>
       </c>
       <c r="M2">
-        <v>0.44309999999999999</v>
+        <v>0.46139999999999998</v>
       </c>
       <c r="N2">
-        <v>28.5366</v>
+        <v>28.841200000000001</v>
       </c>
       <c r="O2">
-        <v>17.219799999999999</v>
+        <v>17.479500000000002</v>
       </c>
       <c r="P2">
-        <v>11.3169</v>
-      </c>
-      <c r="S2">
-        <v>0.42859999999999998</v>
-      </c>
-      <c r="T2">
-        <v>28.956800000000001</v>
-      </c>
-      <c r="U2">
-        <v>17.529399999999999</v>
-      </c>
-      <c r="V2">
-        <v>11.4274</v>
+        <v>11.361700000000001</v>
       </c>
       <c r="X2" t="s">
         <v>40</v>
@@ -2577,28 +2565,16 @@
         <v>10.9596</v>
       </c>
       <c r="M3">
-        <v>0.55689999999999995</v>
+        <v>0.53859999999999997</v>
       </c>
       <c r="N3">
-        <v>21.9603</v>
+        <v>21.1875</v>
       </c>
       <c r="O3">
-        <v>12.2713</v>
+        <v>11.7752</v>
       </c>
       <c r="P3">
-        <v>9.6890000000000001</v>
-      </c>
-      <c r="S3">
-        <v>0.57140000000000002</v>
-      </c>
-      <c r="T3">
-        <v>21.393799999999999</v>
-      </c>
-      <c r="U3">
-        <v>11.8089</v>
-      </c>
-      <c r="V3">
-        <v>9.5847999999999995</v>
+        <v>9.4123000000000001</v>
       </c>
       <c r="X3" t="s">
         <v>41</v>
@@ -2621,28 +2597,16 @@
         <v>5.7394999999999996</v>
       </c>
       <c r="M4">
-        <v>0.68959999999999999</v>
+        <v>0.6966</v>
       </c>
       <c r="N4">
-        <v>30.138300000000001</v>
+        <v>30.259399999999999</v>
       </c>
       <c r="O4">
-        <v>23.950700000000001</v>
+        <v>23.874099999999999</v>
       </c>
       <c r="P4">
-        <v>6.1875</v>
-      </c>
-      <c r="S4">
-        <v>0.67859999999999998</v>
-      </c>
-      <c r="T4">
-        <v>30.261800000000001</v>
-      </c>
-      <c r="U4">
-        <v>23.8552</v>
-      </c>
-      <c r="V4">
-        <v>6.4066000000000001</v>
+        <v>6.3853</v>
       </c>
       <c r="X4" t="s">
         <v>42</v>
@@ -2665,28 +2629,16 @@
         <v>5.9078999999999997</v>
       </c>
       <c r="M5">
-        <v>0.31040000000000001</v>
+        <v>0.3034</v>
       </c>
       <c r="N5">
-        <v>23.289100000000001</v>
+        <v>22.985099999999999</v>
       </c>
       <c r="O5">
-        <v>16.069099999999999</v>
+        <v>16.266100000000002</v>
       </c>
       <c r="P5">
-        <v>7.2199</v>
-      </c>
-      <c r="S5">
-        <v>0.32140000000000002</v>
-      </c>
-      <c r="T5">
-        <v>23.019400000000001</v>
-      </c>
-      <c r="U5">
-        <v>16.190300000000001</v>
-      </c>
-      <c r="V5">
-        <v>6.8291000000000004</v>
+        <v>6.7190000000000003</v>
       </c>
       <c r="X5" t="s">
         <v>43</v>
@@ -2710,35 +2662,23 @@
         <v>4.0126999999999997</v>
       </c>
       <c r="M6">
-        <v>0.93600000000000005</v>
+        <v>0.93440000000000001</v>
       </c>
       <c r="N6">
-        <v>33.424700000000001</v>
+        <v>33.4285</v>
       </c>
       <c r="O6">
-        <v>29.8184</v>
+        <v>29.7196</v>
       </c>
       <c r="P6">
-        <v>3.6063000000000001</v>
-      </c>
-      <c r="S6">
-        <v>0.91590000000000005</v>
-      </c>
-      <c r="T6">
-        <v>33.386800000000001</v>
-      </c>
-      <c r="U6">
-        <v>29.600899999999999</v>
-      </c>
-      <c r="V6">
-        <v>3.7858999999999998</v>
+        <v>3.7088999999999999</v>
       </c>
       <c r="X6" t="s">
         <v>50</v>
       </c>
       <c r="Y6">
         <f>AF21*Y3/100+AJ21*Y4/100+AN21*Y5/100</f>
-        <v>29.300209970200001</v>
+        <v>29.311219341600001</v>
       </c>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
@@ -2755,28 +2695,16 @@
         <v>3.3725999999999998</v>
       </c>
       <c r="M7">
-        <v>6.4000000000000001E-2</v>
+        <v>6.5600000000000006E-2</v>
       </c>
       <c r="N7">
-        <v>23.822600000000001</v>
+        <v>24.541399999999999</v>
       </c>
       <c r="O7">
-        <v>17.418600000000001</v>
+        <v>19.137799999999999</v>
       </c>
       <c r="P7">
-        <v>6.4039999999999999</v>
-      </c>
-      <c r="S7">
-        <v>8.4099999999999994E-2</v>
-      </c>
-      <c r="T7">
-        <v>24.4633</v>
-      </c>
-      <c r="U7">
-        <v>19.1035</v>
-      </c>
-      <c r="V7">
-        <v>5.3597999999999999</v>
+        <v>5.4036</v>
       </c>
     </row>
     <row r="8" spans="1:34" x14ac:dyDescent="0.25">
@@ -2792,36 +2720,12 @@
       <c r="D8">
         <v>11.552</v>
       </c>
-      <c r="M8">
-        <v>0.54879999999999995</v>
-      </c>
-      <c r="N8">
-        <v>30.038399999999999</v>
-      </c>
-      <c r="O8">
-        <v>15.1334</v>
-      </c>
-      <c r="P8">
-        <v>14.904999999999999</v>
-      </c>
-      <c r="S8">
-        <v>0.5544</v>
-      </c>
-      <c r="T8">
-        <v>30.3338</v>
-      </c>
-      <c r="U8">
-        <v>15.0909</v>
-      </c>
-      <c r="V8">
-        <v>15.242900000000001</v>
-      </c>
       <c r="X8" t="s">
         <v>44</v>
       </c>
       <c r="Y8">
         <f>(AD22/100*Y3/100+AH22/100*Y4/100+AL22/100*Y5/100)*100</f>
-        <v>74.379400000000004</v>
+        <v>74.927999999999997</v>
       </c>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
@@ -2837,36 +2741,12 @@
       <c r="D9">
         <v>13.2494</v>
       </c>
-      <c r="M9">
-        <v>0.45119999999999999</v>
-      </c>
-      <c r="N9">
-        <v>23.815100000000001</v>
-      </c>
-      <c r="O9">
-        <v>10.379899999999999</v>
-      </c>
-      <c r="P9">
-        <v>13.4352</v>
-      </c>
-      <c r="S9">
-        <v>0.4456</v>
-      </c>
-      <c r="T9">
-        <v>23.210699999999999</v>
-      </c>
-      <c r="U9">
-        <v>9.9444999999999997</v>
-      </c>
-      <c r="V9">
-        <v>13.2662</v>
-      </c>
       <c r="X9" t="s">
         <v>45</v>
       </c>
       <c r="Y9">
         <f>100-Y8</f>
-        <v>25.620599999999996</v>
+        <v>25.072000000000003</v>
       </c>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
@@ -2882,33 +2762,9 @@
       <c r="D10">
         <v>7.1492000000000004</v>
       </c>
-      <c r="M10">
-        <v>0.72419999999999995</v>
-      </c>
-      <c r="N10">
-        <v>33.209099999999999</v>
-      </c>
-      <c r="O10">
-        <v>26.057200000000002</v>
-      </c>
-      <c r="P10">
-        <v>7.1519000000000004</v>
-      </c>
-      <c r="S10">
-        <v>0.71779999999999999</v>
-      </c>
-      <c r="T10">
-        <v>33.219099999999997</v>
-      </c>
-      <c r="U10">
-        <v>25.819900000000001</v>
-      </c>
-      <c r="V10">
-        <v>7.3992000000000004</v>
-      </c>
       <c r="Y10">
         <f>Y8-Y9</f>
-        <v>48.758800000000008</v>
+        <v>49.855999999999995</v>
       </c>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
@@ -2924,30 +2780,6 @@
       <c r="D11">
         <v>6.9217000000000004</v>
       </c>
-      <c r="M11">
-        <v>0.27579999999999999</v>
-      </c>
-      <c r="N11">
-        <v>25.952400000000001</v>
-      </c>
-      <c r="O11">
-        <v>16.8109</v>
-      </c>
-      <c r="P11">
-        <v>9.1415000000000006</v>
-      </c>
-      <c r="S11">
-        <v>0.28220000000000001</v>
-      </c>
-      <c r="T11">
-        <v>26.0535</v>
-      </c>
-      <c r="U11">
-        <v>17.647300000000001</v>
-      </c>
-      <c r="V11">
-        <v>8.4062000000000001</v>
-      </c>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -2962,36 +2794,12 @@
       <c r="D12">
         <v>4.8164999999999996</v>
       </c>
-      <c r="M12">
-        <v>0.93610000000000004</v>
-      </c>
-      <c r="N12">
-        <v>34.973700000000001</v>
-      </c>
-      <c r="O12">
-        <v>30.670500000000001</v>
-      </c>
-      <c r="P12">
-        <v>4.3032000000000004</v>
-      </c>
-      <c r="S12">
-        <v>0.92710000000000004</v>
-      </c>
-      <c r="T12">
-        <v>34.942599999999999</v>
-      </c>
-      <c r="U12">
-        <v>30.402899999999999</v>
-      </c>
-      <c r="V12">
-        <v>4.5396999999999998</v>
-      </c>
       <c r="X12" t="s">
         <v>46</v>
       </c>
       <c r="Y12">
         <f>AD22/100*Y3/100/(Y8/100)*100</f>
-        <v>8.3402124781861637</v>
+        <v>8.6210762331838566</v>
       </c>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
@@ -3007,36 +2815,12 @@
       <c r="D13">
         <v>4.1228999999999996</v>
       </c>
-      <c r="M13">
-        <v>6.3899999999999998E-2</v>
-      </c>
-      <c r="N13">
-        <v>27.5351</v>
-      </c>
-      <c r="O13">
-        <v>18.8123</v>
-      </c>
-      <c r="P13">
-        <v>8.7227999999999994</v>
-      </c>
-      <c r="S13">
-        <v>7.2900000000000006E-2</v>
-      </c>
-      <c r="T13">
-        <v>28.201499999999999</v>
-      </c>
-      <c r="U13">
-        <v>20.847899999999999</v>
-      </c>
-      <c r="V13">
-        <v>7.3536000000000001</v>
-      </c>
       <c r="X13" t="s">
         <v>47</v>
       </c>
       <c r="Y13">
         <f>AH22/100*Y4/100/(Y8/100)*100</f>
-        <v>46.356921405658014</v>
+        <v>46.484625240230628</v>
       </c>
       <c r="AH13">
         <v>6.2</v>
@@ -3048,7 +2832,7 @@
       </c>
       <c r="Y14">
         <f>100-Y13-Y12</f>
-        <v>45.302866116155826</v>
+        <v>44.894298526585516</v>
       </c>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
@@ -3060,7 +2844,7 @@
       </c>
       <c r="Y15">
         <f>AF22*Y12/100+AJ22*Y13/100+AN22*Y14/100</f>
-        <v>31.49354820877824</v>
+        <v>31.559881111467011</v>
       </c>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
@@ -3103,7 +2887,7 @@
       </c>
       <c r="Y16">
         <f>(Y6-Y8/100*Y15)*100/Y9</f>
-        <v>22.932709514219013</v>
+        <v>22.591064224633051</v>
       </c>
     </row>
     <row r="17" spans="1:46" x14ac:dyDescent="0.25">
@@ -3143,7 +2927,7 @@
       </c>
       <c r="Y17">
         <f>Y15-Y16</f>
-        <v>8.5608386945592265</v>
+        <v>8.9688168868339595</v>
       </c>
     </row>
     <row r="18" spans="1:46" x14ac:dyDescent="0.25">
@@ -3272,28 +3056,28 @@
       </c>
       <c r="O20" s="2">
         <f>M2*100</f>
-        <v>44.31</v>
+        <v>46.14</v>
       </c>
       <c r="P20" t="s">
         <v>3</v>
       </c>
       <c r="Q20" s="2">
         <f>N2</f>
-        <v>28.5366</v>
+        <v>28.841200000000001</v>
       </c>
       <c r="R20" t="s">
         <v>9</v>
       </c>
       <c r="S20" s="2">
         <f>O2</f>
-        <v>17.219799999999999</v>
+        <v>17.479500000000002</v>
       </c>
       <c r="T20" t="s">
         <v>9</v>
       </c>
       <c r="U20" s="2">
         <f>P2</f>
-        <v>11.3169</v>
+        <v>11.361700000000001</v>
       </c>
       <c r="V20" s="3" t="s">
         <v>4</v>
@@ -3408,28 +3192,28 @@
       </c>
       <c r="O21" s="2">
         <f>M3*100</f>
-        <v>55.69</v>
+        <v>53.86</v>
       </c>
       <c r="P21" t="s">
         <v>3</v>
       </c>
       <c r="Q21" s="2">
         <f>N3</f>
-        <v>21.9603</v>
+        <v>21.1875</v>
       </c>
       <c r="R21" t="s">
         <v>9</v>
       </c>
       <c r="S21" s="2">
         <f>O3</f>
-        <v>12.2713</v>
+        <v>11.7752</v>
       </c>
       <c r="T21" t="s">
         <v>9</v>
       </c>
       <c r="U21" s="2">
         <f>P3</f>
-        <v>9.6890000000000001</v>
+        <v>9.4123000000000001</v>
       </c>
       <c r="V21" s="3" t="s">
         <v>4</v>
@@ -3460,7 +3244,7 @@
       </c>
       <c r="AF21" s="2">
         <f>AD22/100*AF22+AD23/100*AF23</f>
-        <v>24.874258529999999</v>
+        <v>24.718917179999998</v>
       </c>
       <c r="AG21" t="s">
         <v>9</v>
@@ -3473,7 +3257,7 @@
       </c>
       <c r="AJ21" s="2">
         <f>AH22/100*AJ22+AH23/100*AJ23</f>
-        <v>28.012308320000002</v>
+        <v>28.052377379999999</v>
       </c>
       <c r="AK21" t="s">
         <v>9</v>
@@ -3486,28 +3270,28 @@
       </c>
       <c r="AN21" s="2">
         <f>AL22/100*AN22+AL23/100*AN23</f>
-        <v>32.810165599999998</v>
+        <v>32.845506239999999</v>
       </c>
       <c r="AO21" t="s">
         <v>3</v>
       </c>
       <c r="AP21" s="2">
         <f>AN21-AF21</f>
-        <v>7.935907069999999</v>
+        <v>8.1265890600000006</v>
       </c>
       <c r="AQ21" t="s">
         <v>3</v>
       </c>
       <c r="AR21" s="2">
         <f>AN21-(AF22*AL22/100+AF23*AL23/100)</f>
-        <v>4.6944488</v>
+        <v>4.5063889599999989</v>
       </c>
       <c r="AS21" s="3" t="s">
         <v>4</v>
       </c>
       <c r="AT21" s="7">
         <f>(AP21-AR21)/AP21</f>
-        <v>0.40845466578781392</v>
+        <v>0.44547596454938765</v>
       </c>
     </row>
     <row r="22" spans="1:46" x14ac:dyDescent="0.25">
@@ -3552,28 +3336,28 @@
       </c>
       <c r="O22" s="2">
         <f>O20-O21</f>
-        <v>-11.379999999999995</v>
+        <v>-7.7199999999999989</v>
       </c>
       <c r="P22" t="s">
         <v>3</v>
       </c>
       <c r="Q22" s="2">
         <f>Q20-Q21</f>
-        <v>6.5762999999999998</v>
+        <v>7.6537000000000006</v>
       </c>
       <c r="R22" t="s">
         <v>9</v>
       </c>
       <c r="S22" s="2">
         <f>S20-S21</f>
-        <v>4.9484999999999992</v>
+        <v>5.7043000000000017</v>
       </c>
       <c r="T22" t="s">
         <v>9</v>
       </c>
       <c r="U22" s="2">
         <f>U20-U21</f>
-        <v>1.6279000000000003</v>
+        <v>1.9494000000000007</v>
       </c>
       <c r="V22" s="3" t="s">
         <v>4</v>
@@ -3598,49 +3382,49 @@
       </c>
       <c r="AD22" s="2">
         <f>100-AD23</f>
-        <v>44.31</v>
+        <v>46.14</v>
       </c>
       <c r="AE22" t="s">
         <v>3</v>
       </c>
       <c r="AF22" s="2">
         <f>Q20</f>
-        <v>28.5366</v>
+        <v>28.841200000000001</v>
       </c>
       <c r="AG22" t="s">
         <v>9</v>
       </c>
       <c r="AH22" s="2">
         <f>O26</f>
-        <v>68.959999999999994</v>
+        <v>69.66</v>
       </c>
       <c r="AI22" t="s">
         <v>3</v>
       </c>
       <c r="AJ22" s="2">
         <f>Q26</f>
-        <v>30.138300000000001</v>
+        <v>30.259399999999999</v>
       </c>
       <c r="AK22" t="s">
         <v>9</v>
       </c>
       <c r="AL22" s="2">
         <f>100-AL23</f>
-        <v>93.6</v>
+        <v>93.44</v>
       </c>
       <c r="AM22" t="s">
         <v>3</v>
       </c>
       <c r="AN22" s="2">
         <f>Q32</f>
-        <v>33.424700000000001</v>
+        <v>33.4285</v>
       </c>
       <c r="AO22" t="s">
         <v>3</v>
       </c>
       <c r="AP22" s="2">
         <f t="shared" ref="AP22:AP24" si="0">AN22-AF22</f>
-        <v>4.8881000000000014</v>
+        <v>4.587299999999999</v>
       </c>
       <c r="AQ22" t="s">
         <v>3</v>
@@ -3673,21 +3457,21 @@
       </c>
       <c r="Q23">
         <f>ROUND(Q20*$O20/100+Q21*$O21/100,1)</f>
-        <v>24.9</v>
+        <v>24.7</v>
       </c>
       <c r="R23" t="s">
         <v>9</v>
       </c>
       <c r="S23">
         <f>ROUND(S20*$O20/100+S21*$O21/100,1)</f>
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="T23" t="s">
         <v>9</v>
       </c>
       <c r="U23">
         <f>ROUND(U20*$O20/100+U21*$O21/100,1)</f>
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="V23" s="3" t="s">
         <v>4</v>
@@ -3712,49 +3496,49 @@
       </c>
       <c r="AD23" s="2">
         <f>O21</f>
-        <v>55.69</v>
+        <v>53.86</v>
       </c>
       <c r="AE23" t="s">
         <v>3</v>
       </c>
       <c r="AF23" s="2">
         <f>Q21</f>
-        <v>21.9603</v>
+        <v>21.1875</v>
       </c>
       <c r="AG23" t="s">
         <v>9</v>
       </c>
       <c r="AH23" s="2">
         <f>O27</f>
-        <v>31.04</v>
+        <v>30.34</v>
       </c>
       <c r="AI23" t="s">
         <v>3</v>
       </c>
       <c r="AJ23" s="2">
         <f>Q27</f>
-        <v>23.289100000000001</v>
+        <v>22.985099999999999</v>
       </c>
       <c r="AK23" t="s">
         <v>9</v>
       </c>
       <c r="AL23" s="2">
         <f>O33</f>
-        <v>6.4</v>
+        <v>6.5600000000000005</v>
       </c>
       <c r="AM23" t="s">
         <v>3</v>
       </c>
       <c r="AN23" s="2">
         <f>Q33</f>
-        <v>23.822600000000001</v>
+        <v>24.541399999999999</v>
       </c>
       <c r="AO23" t="s">
         <v>3</v>
       </c>
       <c r="AP23" s="2">
         <f t="shared" si="0"/>
-        <v>1.8623000000000012</v>
+        <v>3.3538999999999994</v>
       </c>
       <c r="AQ23" t="s">
         <v>3</v>
@@ -3809,14 +3593,14 @@
       </c>
       <c r="Q24">
         <f>ROUND(Q20*$O$32/100+Q21*$O$33/100,1)</f>
-        <v>28.1</v>
+        <v>28.3</v>
       </c>
       <c r="R24" t="s">
         <v>9</v>
       </c>
       <c r="S24" s="2">
         <f>ROUND(S20*$O$32/100+S21*$O$33/100,1)</f>
-        <v>16.899999999999999</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="T24" t="s">
         <v>9</v>
@@ -3848,49 +3632,49 @@
       </c>
       <c r="AD24" s="2">
         <f>AD22-AD23</f>
-        <v>-11.379999999999995</v>
+        <v>-7.7199999999999989</v>
       </c>
       <c r="AE24" t="s">
         <v>3</v>
       </c>
       <c r="AF24" s="2">
         <f>AF22-AF23</f>
-        <v>6.5762999999999998</v>
+        <v>7.6537000000000006</v>
       </c>
       <c r="AG24" t="s">
         <v>9</v>
       </c>
       <c r="AH24" s="2">
         <f>AH22-AH23</f>
-        <v>37.919999999999995</v>
+        <v>39.319999999999993</v>
       </c>
       <c r="AI24" t="s">
         <v>3</v>
       </c>
       <c r="AJ24" s="2">
         <f>AJ22-AJ23</f>
-        <v>6.8491999999999997</v>
+        <v>7.2743000000000002</v>
       </c>
       <c r="AK24" t="s">
         <v>9</v>
       </c>
       <c r="AL24" s="2">
         <f>AL22-AL23</f>
-        <v>87.199999999999989</v>
+        <v>86.88</v>
       </c>
       <c r="AM24" t="s">
         <v>3</v>
       </c>
       <c r="AN24" s="2">
         <f>AN22-AN23</f>
-        <v>9.6021000000000001</v>
+        <v>8.8871000000000002</v>
       </c>
       <c r="AO24" t="s">
         <v>3</v>
       </c>
       <c r="AP24" s="2">
         <f t="shared" si="0"/>
-        <v>3.0258000000000003</v>
+        <v>1.2333999999999996</v>
       </c>
       <c r="AQ24" t="s">
         <v>3</v>
@@ -3987,28 +3771,28 @@
       </c>
       <c r="O26" s="2">
         <f>M4*100</f>
-        <v>68.959999999999994</v>
+        <v>69.66</v>
       </c>
       <c r="P26" t="s">
         <v>3</v>
       </c>
       <c r="Q26" s="2">
         <f>N4</f>
-        <v>30.138300000000001</v>
+        <v>30.259399999999999</v>
       </c>
       <c r="R26" t="s">
         <v>9</v>
       </c>
       <c r="S26" s="2">
         <f>O4</f>
-        <v>23.950700000000001</v>
+        <v>23.874099999999999</v>
       </c>
       <c r="T26" t="s">
         <v>9</v>
       </c>
       <c r="U26" s="2">
         <f>P4</f>
-        <v>6.1875</v>
+        <v>6.3853</v>
       </c>
       <c r="V26" s="3" t="s">
         <v>4</v>
@@ -4036,28 +3820,28 @@
       </c>
       <c r="O27" s="2">
         <f>M5*100</f>
-        <v>31.04</v>
+        <v>30.34</v>
       </c>
       <c r="P27" t="s">
         <v>3</v>
       </c>
       <c r="Q27" s="2">
         <f>N5</f>
-        <v>23.289100000000001</v>
+        <v>22.985099999999999</v>
       </c>
       <c r="R27" t="s">
         <v>9</v>
       </c>
       <c r="S27" s="2">
         <f>O5</f>
-        <v>16.069099999999999</v>
+        <v>16.266100000000002</v>
       </c>
       <c r="T27" t="s">
         <v>9</v>
       </c>
       <c r="U27" s="2">
         <f>P5</f>
-        <v>7.2199</v>
+        <v>6.7190000000000003</v>
       </c>
       <c r="V27" s="3" t="s">
         <v>4</v>
@@ -4111,28 +3895,28 @@
       </c>
       <c r="O28" s="2">
         <f>O26-O27</f>
-        <v>37.919999999999995</v>
+        <v>39.319999999999993</v>
       </c>
       <c r="P28" t="s">
         <v>3</v>
       </c>
       <c r="Q28" s="2">
         <f>Q26-Q27</f>
-        <v>6.8491999999999997</v>
+        <v>7.2743000000000002</v>
       </c>
       <c r="R28" t="s">
         <v>9</v>
       </c>
       <c r="S28" s="2">
         <f>S26-S27</f>
-        <v>7.8816000000000024</v>
+        <v>7.607999999999997</v>
       </c>
       <c r="T28" t="s">
         <v>9</v>
       </c>
       <c r="U28" s="2">
         <f>U26-U27</f>
-        <v>-1.0324</v>
+        <v>-0.33370000000000033</v>
       </c>
       <c r="V28" s="3" t="s">
         <v>4</v>
@@ -4192,14 +3976,14 @@
       </c>
       <c r="Q29">
         <f>ROUND(Q26*$O26/100+Q27*$O27/100,1)</f>
-        <v>28</v>
+        <v>28.1</v>
       </c>
       <c r="R29" t="s">
         <v>9</v>
       </c>
       <c r="S29">
         <f>ROUND(S26*$O26/100+S27*$O27/100,1)</f>
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="T29" t="s">
         <v>9</v>
@@ -4257,7 +4041,7 @@
       </c>
       <c r="Q30">
         <f>ROUND(Q26*$O$32/100+Q27*$O$33/100,1)</f>
-        <v>29.7</v>
+        <v>29.8</v>
       </c>
       <c r="R30" t="s">
         <v>9</v>
@@ -4271,7 +4055,7 @@
       </c>
       <c r="U30">
         <f>ROUND(U26*$O$32/100+U27*$O$33/100,1)</f>
-        <v>6.3</v>
+        <v>6.4</v>
       </c>
       <c r="V30" t="s">
         <v>27</v>
@@ -4365,28 +4149,28 @@
       </c>
       <c r="O32" s="2">
         <f>M6*100</f>
-        <v>93.600000000000009</v>
+        <v>93.44</v>
       </c>
       <c r="P32" t="s">
         <v>3</v>
       </c>
       <c r="Q32" s="2">
         <f>N6</f>
-        <v>33.424700000000001</v>
+        <v>33.4285</v>
       </c>
       <c r="R32" t="s">
         <v>9</v>
       </c>
       <c r="S32" s="2">
         <f>O6</f>
-        <v>29.8184</v>
+        <v>29.7196</v>
       </c>
       <c r="T32" t="s">
         <v>9</v>
       </c>
       <c r="U32" s="2">
         <f>P6</f>
-        <v>3.6063000000000001</v>
+        <v>3.7088999999999999</v>
       </c>
       <c r="V32" s="3" t="s">
         <v>4</v>
@@ -4489,28 +4273,28 @@
       </c>
       <c r="O33" s="2">
         <f>M7*100</f>
-        <v>6.4</v>
+        <v>6.5600000000000005</v>
       </c>
       <c r="P33" t="s">
         <v>3</v>
       </c>
       <c r="Q33" s="2">
         <f>N7</f>
-        <v>23.822600000000001</v>
+        <v>24.541399999999999</v>
       </c>
       <c r="R33" t="s">
         <v>9</v>
       </c>
       <c r="S33" s="2">
         <f>O7</f>
-        <v>17.418600000000001</v>
+        <v>19.137799999999999</v>
       </c>
       <c r="T33" t="s">
         <v>9</v>
       </c>
       <c r="U33" s="2">
         <f>P7</f>
-        <v>6.4039999999999999</v>
+        <v>5.4036</v>
       </c>
       <c r="V33" s="3" t="s">
         <v>4</v>
@@ -4529,7 +4313,7 @@
       </c>
       <c r="AB33" s="2">
         <f>Z34/100*AB34+Z35/100*AB35</f>
-        <v>27.230447039999998</v>
+        <v>0</v>
       </c>
       <c r="AC33" t="s">
         <v>9</v>
@@ -4542,7 +4326,7 @@
       </c>
       <c r="AF33" s="2">
         <f>AD34/100*AF34+AD35/100*AF35</f>
-        <v>31.207702140000002</v>
+        <v>0</v>
       </c>
       <c r="AG33" t="s">
         <v>9</v>
@@ -4555,28 +4339,28 @@
       </c>
       <c r="AJ33" s="2">
         <f>AH34/100*AJ34+AH35/100*AJ35</f>
-        <v>34.498373459999996</v>
+        <v>0</v>
       </c>
       <c r="AK33" t="s">
         <v>3</v>
       </c>
       <c r="AL33" s="2">
         <f>AJ33-AB33</f>
-        <v>7.2679264199999984</v>
+        <v>0</v>
       </c>
       <c r="AM33" t="s">
         <v>3</v>
       </c>
       <c r="AN33" s="2">
         <f>AJ33-(AB34*AH34/100+AB35*AH35/100)</f>
-        <v>4.8576423299999973</v>
+        <v>0</v>
       </c>
       <c r="AO33" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="AP33" s="7">
+      <c r="AP33" s="7" t="e">
         <f>(AL33-AN33)/AL33</f>
-        <v>0.33163297902512362</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="34" spans="1:42" x14ac:dyDescent="0.25">
@@ -4621,28 +4405,28 @@
       </c>
       <c r="O34" s="2">
         <f>O32-O33</f>
-        <v>87.2</v>
+        <v>86.88</v>
       </c>
       <c r="P34" t="s">
         <v>3</v>
       </c>
       <c r="Q34" s="2">
         <f>Q32-Q33</f>
-        <v>9.6021000000000001</v>
+        <v>8.8871000000000002</v>
       </c>
       <c r="R34" t="s">
         <v>9</v>
       </c>
       <c r="S34" s="2">
         <f>S32-S33</f>
-        <v>12.399799999999999</v>
+        <v>10.581800000000001</v>
       </c>
       <c r="T34" t="s">
         <v>9</v>
       </c>
       <c r="U34" s="2">
         <f>U32-U33</f>
-        <v>-2.7976999999999999</v>
+        <v>-1.6947000000000001</v>
       </c>
       <c r="V34" s="3" t="s">
         <v>4</v>
@@ -4655,49 +4439,49 @@
       </c>
       <c r="Z34" s="2">
         <f>O38</f>
-        <v>54.879999999999995</v>
+        <v>0</v>
       </c>
       <c r="AA34" t="s">
         <v>3</v>
       </c>
       <c r="AB34" s="2">
         <f>Q38</f>
-        <v>30.038399999999999</v>
+        <v>0</v>
       </c>
       <c r="AC34" t="s">
         <v>9</v>
       </c>
       <c r="AD34" s="2">
         <f>O44</f>
-        <v>72.42</v>
+        <v>0</v>
       </c>
       <c r="AE34" t="s">
         <v>3</v>
       </c>
       <c r="AF34" s="2">
         <f>Q44</f>
-        <v>33.209099999999999</v>
+        <v>0</v>
       </c>
       <c r="AG34" t="s">
         <v>9</v>
       </c>
       <c r="AH34" s="2">
         <f>O50</f>
-        <v>93.61</v>
+        <v>0</v>
       </c>
       <c r="AI34" t="s">
         <v>3</v>
       </c>
       <c r="AJ34" s="2">
         <f>Q50</f>
-        <v>34.973700000000001</v>
+        <v>0</v>
       </c>
       <c r="AK34" t="s">
         <v>3</v>
       </c>
       <c r="AL34" s="2">
         <f t="shared" ref="AL34:AL35" si="1">AJ34-AB34</f>
-        <v>4.9353000000000016</v>
+        <v>0</v>
       </c>
       <c r="AM34" t="s">
         <v>3</v>
@@ -4756,49 +4540,49 @@
       </c>
       <c r="Z35" s="2">
         <f>O39</f>
-        <v>45.12</v>
+        <v>0</v>
       </c>
       <c r="AA35" t="s">
         <v>3</v>
       </c>
       <c r="AB35" s="2">
         <f>Q39</f>
-        <v>23.815100000000001</v>
+        <v>0</v>
       </c>
       <c r="AC35" t="s">
         <v>9</v>
       </c>
       <c r="AD35" s="2">
         <f>O45</f>
-        <v>27.58</v>
+        <v>0</v>
       </c>
       <c r="AE35" t="s">
         <v>3</v>
       </c>
       <c r="AF35" s="2">
         <f>Q45</f>
-        <v>25.952400000000001</v>
+        <v>0</v>
       </c>
       <c r="AG35" t="s">
         <v>9</v>
       </c>
       <c r="AH35" s="2">
         <f>O51</f>
-        <v>6.39</v>
+        <v>0</v>
       </c>
       <c r="AI35" t="s">
         <v>3</v>
       </c>
       <c r="AJ35" s="2">
         <f>Q51</f>
-        <v>27.5351</v>
+        <v>0</v>
       </c>
       <c r="AK35" t="s">
         <v>3</v>
       </c>
       <c r="AL35" s="2">
         <f t="shared" si="1"/>
-        <v>3.7199999999999989</v>
+        <v>0</v>
       </c>
       <c r="AM35" t="s">
         <v>3</v>
@@ -4880,49 +4664,49 @@
       </c>
       <c r="Z36" s="2">
         <f>Z34-Z35</f>
-        <v>9.759999999999998</v>
+        <v>0</v>
       </c>
       <c r="AA36" t="s">
         <v>3</v>
       </c>
       <c r="AB36" s="2">
         <f>AB34-AB35</f>
-        <v>6.2232999999999983</v>
+        <v>0</v>
       </c>
       <c r="AC36" t="s">
         <v>9</v>
       </c>
       <c r="AD36" s="2">
         <f>AD34-AD35</f>
-        <v>44.84</v>
+        <v>0</v>
       </c>
       <c r="AE36" t="s">
         <v>3</v>
       </c>
       <c r="AF36" s="2">
         <f>AF34-AF35</f>
-        <v>7.2566999999999986</v>
+        <v>0</v>
       </c>
       <c r="AG36" t="s">
         <v>9</v>
       </c>
       <c r="AH36" s="2">
         <f>AH34-AH35</f>
-        <v>87.22</v>
+        <v>0</v>
       </c>
       <c r="AI36" t="s">
         <v>3</v>
       </c>
       <c r="AJ36" s="2">
         <f>AJ34-AJ35</f>
-        <v>7.438600000000001</v>
+        <v>0</v>
       </c>
       <c r="AK36" t="s">
         <v>3</v>
       </c>
       <c r="AL36" s="2">
         <f>AJ36-AB36</f>
-        <v>1.2153000000000027</v>
+        <v>0</v>
       </c>
       <c r="AM36" t="s">
         <v>3</v>
@@ -5022,28 +4806,28 @@
       </c>
       <c r="O38" s="2">
         <f>M8*100</f>
-        <v>54.879999999999995</v>
+        <v>0</v>
       </c>
       <c r="P38" t="s">
         <v>3</v>
       </c>
       <c r="Q38" s="2">
         <f>N8</f>
-        <v>30.038399999999999</v>
+        <v>0</v>
       </c>
       <c r="R38" t="s">
         <v>9</v>
       </c>
       <c r="S38" s="2">
         <f>O8</f>
-        <v>15.1334</v>
+        <v>0</v>
       </c>
       <c r="T38" t="s">
         <v>9</v>
       </c>
       <c r="U38" s="2">
         <f>P8</f>
-        <v>14.904999999999999</v>
+        <v>0</v>
       </c>
       <c r="V38" s="3" t="s">
         <v>4</v>
@@ -5054,15 +4838,15 @@
       <c r="AA38" s="2"/>
       <c r="AB38" s="2">
         <f>AB33-AF21</f>
-        <v>2.3561885099999991</v>
+        <v>-24.718917179999998</v>
       </c>
       <c r="AF38" s="2">
         <f>AF33-AJ21</f>
-        <v>3.1953938199999996</v>
+        <v>-28.052377379999999</v>
       </c>
       <c r="AJ38" s="2">
         <f>AJ33-AN21</f>
-        <v>1.6882078599999986</v>
+        <v>-32.845506239999999</v>
       </c>
     </row>
     <row r="39" spans="1:42" x14ac:dyDescent="0.25">
@@ -5075,28 +4859,28 @@
       </c>
       <c r="O39" s="2">
         <f>M9*100</f>
-        <v>45.12</v>
+        <v>0</v>
       </c>
       <c r="P39" t="s">
         <v>3</v>
       </c>
       <c r="Q39" s="2">
         <f>N9</f>
-        <v>23.815100000000001</v>
+        <v>0</v>
       </c>
       <c r="R39" t="s">
         <v>9</v>
       </c>
       <c r="S39" s="2">
         <f>O9</f>
-        <v>10.379899999999999</v>
+        <v>0</v>
       </c>
       <c r="T39" t="s">
         <v>9</v>
       </c>
       <c r="U39" s="2">
         <f>P9</f>
-        <v>13.4352</v>
+        <v>0</v>
       </c>
       <c r="V39" s="3" t="s">
         <v>4</v>
@@ -5104,7 +4888,7 @@
       <c r="X39" s="2"/>
       <c r="AB39">
         <f>AF22*Z34/100+AF23*Z35/100</f>
-        <v>25.569373439999996</v>
+        <v>0</v>
       </c>
       <c r="AF39" s="2"/>
       <c r="AJ39" s="2"/>
@@ -5118,35 +4902,35 @@
       </c>
       <c r="O40" s="2">
         <f>O38-O39</f>
-        <v>9.759999999999998</v>
+        <v>0</v>
       </c>
       <c r="P40" t="s">
         <v>3</v>
       </c>
       <c r="Q40" s="2">
         <f>Q38-Q39</f>
-        <v>6.2232999999999983</v>
+        <v>0</v>
       </c>
       <c r="R40" t="s">
         <v>9</v>
       </c>
       <c r="S40" s="2">
         <f>S38-S39</f>
-        <v>4.7535000000000007</v>
+        <v>0</v>
       </c>
       <c r="T40" t="s">
         <v>9</v>
       </c>
       <c r="U40" s="2">
         <f>U38-U39</f>
-        <v>1.4697999999999993</v>
+        <v>0</v>
       </c>
       <c r="V40" s="3" t="s">
         <v>4</v>
       </c>
       <c r="AB40" s="2">
         <f>AB33-AB39</f>
-        <v>1.6610736000000017</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:42" x14ac:dyDescent="0.25">
@@ -5164,21 +4948,21 @@
       </c>
       <c r="Q41">
         <f>ROUND(Q38*$O38/100+Q39*$O39/100,1)</f>
-        <v>27.2</v>
+        <v>0</v>
       </c>
       <c r="R41" t="s">
         <v>9</v>
       </c>
       <c r="S41">
         <f>ROUND(S38*$O38/100+S39*$O39/100,1)</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="T41" t="s">
         <v>9</v>
       </c>
       <c r="U41">
         <f>ROUND(U38*$O38/100+U39*$O39/100,1)</f>
-        <v>14.2</v>
+        <v>0</v>
       </c>
       <c r="V41" s="3" t="s">
         <v>4</v>
@@ -5196,21 +4980,21 @@
       </c>
       <c r="Q42">
         <f>ROUND(Q38*$O$50/100+Q39*$O$51/100,1)</f>
-        <v>29.6</v>
+        <v>0</v>
       </c>
       <c r="R42" t="s">
         <v>9</v>
       </c>
       <c r="S42">
         <f>ROUND(S38*$O$50/100+S39*$O$51/100,1)</f>
-        <v>14.8</v>
+        <v>0</v>
       </c>
       <c r="T42" t="s">
         <v>9</v>
       </c>
       <c r="U42">
         <f>ROUND(U38*$O$50/100+U39*$O$51/100,1)</f>
-        <v>14.8</v>
+        <v>0</v>
       </c>
       <c r="V42" t="s">
         <v>27</v>
@@ -5235,28 +5019,28 @@
       </c>
       <c r="O44" s="2">
         <f>M10*100</f>
-        <v>72.42</v>
+        <v>0</v>
       </c>
       <c r="P44" t="s">
         <v>3</v>
       </c>
       <c r="Q44" s="2">
         <f>N10</f>
-        <v>33.209099999999999</v>
+        <v>0</v>
       </c>
       <c r="R44" t="s">
         <v>9</v>
       </c>
       <c r="S44" s="2">
         <f>O10</f>
-        <v>26.057200000000002</v>
+        <v>0</v>
       </c>
       <c r="T44" t="s">
         <v>9</v>
       </c>
       <c r="U44" s="2">
         <f>P10</f>
-        <v>7.1519000000000004</v>
+        <v>0</v>
       </c>
       <c r="V44" s="3" t="s">
         <v>4</v>
@@ -5271,28 +5055,28 @@
       </c>
       <c r="O45" s="2">
         <f>M11*100</f>
-        <v>27.58</v>
+        <v>0</v>
       </c>
       <c r="P45" t="s">
         <v>3</v>
       </c>
       <c r="Q45" s="2">
         <f>N11</f>
-        <v>25.952400000000001</v>
+        <v>0</v>
       </c>
       <c r="R45" t="s">
         <v>9</v>
       </c>
       <c r="S45" s="2">
         <f>O11</f>
-        <v>16.8109</v>
+        <v>0</v>
       </c>
       <c r="T45" t="s">
         <v>9</v>
       </c>
       <c r="U45" s="2">
         <f>P11</f>
-        <v>9.1415000000000006</v>
+        <v>0</v>
       </c>
       <c r="V45" s="3" t="s">
         <v>4</v>
@@ -5307,28 +5091,28 @@
       </c>
       <c r="O46" s="2">
         <f>O44-O45</f>
-        <v>44.84</v>
+        <v>0</v>
       </c>
       <c r="P46" t="s">
         <v>3</v>
       </c>
       <c r="Q46" s="2">
         <f>Q44-Q45</f>
-        <v>7.2566999999999986</v>
+        <v>0</v>
       </c>
       <c r="R46" t="s">
         <v>9</v>
       </c>
       <c r="S46" s="2">
         <f>S44-S45</f>
-        <v>9.2463000000000015</v>
+        <v>0</v>
       </c>
       <c r="T46" t="s">
         <v>9</v>
       </c>
       <c r="U46" s="2">
         <f>U44-U45</f>
-        <v>-1.9896000000000003</v>
+        <v>0</v>
       </c>
       <c r="V46" s="3" t="s">
         <v>4</v>
@@ -5352,21 +5136,21 @@
       </c>
       <c r="Q47">
         <f>ROUND(Q44*$O44/100+Q45*$O45/100,1)</f>
-        <v>31.2</v>
+        <v>0</v>
       </c>
       <c r="R47" t="s">
         <v>9</v>
       </c>
       <c r="S47">
         <f>ROUND(S44*$O44/100+S45*$O45/100,1)</f>
-        <v>23.5</v>
+        <v>0</v>
       </c>
       <c r="T47" t="s">
         <v>9</v>
       </c>
       <c r="U47">
         <f>ROUND(U44*$O44/100+U45*$O45/100,1)</f>
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="V47" s="3" t="s">
         <v>4</v>
@@ -5391,21 +5175,21 @@
       </c>
       <c r="Q48">
         <f>ROUND(Q44*$O$50/100+Q45*$O$51/100,1)</f>
-        <v>32.700000000000003</v>
+        <v>0</v>
       </c>
       <c r="R48" t="s">
         <v>9</v>
       </c>
       <c r="S48">
         <f>ROUND(S44*$O$50/100+S45*$O$51/100,1)</f>
-        <v>25.5</v>
+        <v>0</v>
       </c>
       <c r="T48" t="s">
         <v>9</v>
       </c>
       <c r="U48">
         <f>ROUND(U44*$O$50/100+U45*$O$51/100,1)</f>
-        <v>7.3</v>
+        <v>0</v>
       </c>
       <c r="V48" t="s">
         <v>27</v>
@@ -5423,9 +5207,9 @@
       <c r="S49" s="2"/>
       <c r="U49" s="2"/>
       <c r="V49" s="3"/>
-      <c r="X49" s="5">
+      <c r="X49" s="5" t="e">
         <f>(X38-Q40)/(Q52-Q40)</f>
-        <v>-5.1207932197811115</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="Y49" s="5"/>
       <c r="Z49" s="5"/>
@@ -5442,28 +5226,28 @@
       </c>
       <c r="O50" s="2">
         <f>M12*100</f>
-        <v>93.61</v>
+        <v>0</v>
       </c>
       <c r="P50" t="s">
         <v>3</v>
       </c>
       <c r="Q50" s="2">
         <f>N12</f>
-        <v>34.973700000000001</v>
+        <v>0</v>
       </c>
       <c r="R50" t="s">
         <v>9</v>
       </c>
       <c r="S50" s="2">
         <f>O12</f>
-        <v>30.670500000000001</v>
+        <v>0</v>
       </c>
       <c r="T50" t="s">
         <v>9</v>
       </c>
       <c r="U50" s="2">
         <f>P12</f>
-        <v>4.3032000000000004</v>
+        <v>0</v>
       </c>
       <c r="V50" s="3" t="s">
         <v>4</v>
@@ -5481,28 +5265,28 @@
       </c>
       <c r="O51" s="2">
         <f>M13*100</f>
-        <v>6.39</v>
+        <v>0</v>
       </c>
       <c r="P51" t="s">
         <v>3</v>
       </c>
       <c r="Q51" s="2">
         <f>N13</f>
-        <v>27.5351</v>
+        <v>0</v>
       </c>
       <c r="R51" t="s">
         <v>9</v>
       </c>
       <c r="S51" s="2">
         <f>O13</f>
-        <v>18.8123</v>
+        <v>0</v>
       </c>
       <c r="T51" t="s">
         <v>9</v>
       </c>
       <c r="U51" s="2">
         <f>P13</f>
-        <v>8.7227999999999994</v>
+        <v>0</v>
       </c>
       <c r="V51" s="3" t="s">
         <v>4</v>
@@ -5520,28 +5304,28 @@
       </c>
       <c r="O52" s="2">
         <f>O50-O51</f>
-        <v>87.22</v>
+        <v>0</v>
       </c>
       <c r="P52" t="s">
         <v>3</v>
       </c>
       <c r="Q52" s="2">
         <f>Q50-Q51</f>
-        <v>7.438600000000001</v>
+        <v>0</v>
       </c>
       <c r="R52" t="s">
         <v>9</v>
       </c>
       <c r="S52" s="2">
         <f>S50-S51</f>
-        <v>11.8582</v>
+        <v>0</v>
       </c>
       <c r="T52" t="s">
         <v>9</v>
       </c>
       <c r="U52" s="2">
         <f>U50-U51</f>
-        <v>-4.4195999999999991</v>
+        <v>0</v>
       </c>
       <c r="V52" s="3" t="s">
         <v>4</v>
@@ -5565,21 +5349,21 @@
       </c>
       <c r="Q53">
         <f>ROUND(Q50*$O50/100+Q51*$O51/100,1)</f>
-        <v>34.5</v>
+        <v>0</v>
       </c>
       <c r="R53" t="s">
         <v>9</v>
       </c>
       <c r="S53">
         <f>ROUND(S50*$O50/100+S51*$O51/100,1)</f>
-        <v>29.9</v>
+        <v>0</v>
       </c>
       <c r="T53" t="s">
         <v>9</v>
       </c>
       <c r="U53">
         <f>ROUND(U50*$O50/100+U51*$O51/100,1)</f>
-        <v>4.5999999999999996</v>
+        <v>0</v>
       </c>
       <c r="V53" s="3" t="s">
         <v>4</v>
@@ -5598,21 +5382,21 @@
       </c>
       <c r="Q54">
         <f>ROUND(Q50*$O$50/100+Q51*$O$51/100,1)</f>
-        <v>34.5</v>
+        <v>0</v>
       </c>
       <c r="R54" t="s">
         <v>9</v>
       </c>
       <c r="S54">
         <f>ROUND(S50*$O$50/100+S51*$O$51/100,1)</f>
-        <v>29.9</v>
+        <v>0</v>
       </c>
       <c r="T54" t="s">
         <v>9</v>
       </c>
       <c r="U54">
         <f>ROUND(U50*$O$50/100+U51*$O$51/100,1)</f>
-        <v>4.5999999999999996</v>
+        <v>0</v>
       </c>
       <c r="V54" s="3" t="s">
         <v>36</v>

</xml_diff>